<commit_message>
Nuovo ordine_template.xlsx + niente cache CDN sul template di lavoro
</commit_message>
<xml_diff>
--- a/ordine_template.xlsx
+++ b/ordine_template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC_Graphic\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GRAFICA\GRAFICA 2026\programma occhiali detomaso\09 09 2026 inserimento 3 NUOVI ARTICOLI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A54806A9-E677-4C33-A913-2BC90280081B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7DE9FA84-36F5-4EB6-A9ED-AAD402438EDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{1DF05D46-8AE3-4E7B-8533-2DA2E4746004}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2586" uniqueCount="708">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2577" uniqueCount="707">
   <si>
     <t>CODICE</t>
   </si>
@@ -2100,9 +2100,6 @@
   </si>
   <si>
     <t>PROVINCIA:</t>
-  </si>
-  <si>
-    <t>OBBLIGATORIO</t>
   </si>
   <si>
     <t>CELLULARE:</t>
@@ -2631,7 +2628,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="97">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
@@ -2797,6 +2794,43 @@
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -2808,21 +2842,6 @@
     <xf numFmtId="0" fontId="9" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="5" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="5" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="6" fillId="6" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="12" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2841,30 +2860,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="12" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2914,44 +2909,19 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="5" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="10" fontId="5" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="44" fontId="6" fillId="6" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3294,274 +3264,256 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:20" s="1" customFormat="1" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="84" t="s">
+      <c r="A2" s="53" t="s">
         <v>367</v>
       </c>
-      <c r="B2" s="85"/>
-      <c r="C2" s="85"/>
-      <c r="D2" s="85"/>
-      <c r="E2" s="85"/>
-      <c r="F2" s="85"/>
-      <c r="G2" s="85"/>
-      <c r="H2" s="85"/>
-      <c r="I2" s="85"/>
-      <c r="J2" s="85"/>
-      <c r="K2" s="85"/>
-      <c r="L2" s="85"/>
-      <c r="M2" s="85"/>
-      <c r="N2" s="85"/>
-      <c r="O2" s="85"/>
-      <c r="P2" s="85"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="54"/>
+      <c r="J2" s="54"/>
+      <c r="K2" s="54"/>
+      <c r="L2" s="54"/>
+      <c r="M2" s="54"/>
+      <c r="N2" s="54"/>
+      <c r="O2" s="54"/>
+      <c r="P2" s="54"/>
       <c r="R2" s="2"/>
     </row>
     <row r="3" spans="1:20" s="1" customFormat="1" ht="6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="R3" s="2"/>
     </row>
     <row r="4" spans="1:20" s="1" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="67" t="s">
+      <c r="A4" s="60" t="s">
         <v>686</v>
       </c>
-      <c r="B4" s="68"/>
-      <c r="C4" s="68"/>
-      <c r="D4" s="66" t="s">
-        <v>688</v>
-      </c>
-      <c r="E4" s="66"/>
-      <c r="F4" s="66"/>
-      <c r="G4" s="66"/>
+      <c r="B4" s="61"/>
+      <c r="C4" s="61"/>
+      <c r="D4" s="59"/>
+      <c r="E4" s="59"/>
+      <c r="F4" s="59"/>
+      <c r="G4" s="59"/>
       <c r="H4" s="3" t="s">
         <v>368</v>
       </c>
-      <c r="I4" s="52"/>
-      <c r="J4" s="53"/>
-      <c r="K4" s="53"/>
-      <c r="L4" s="53"/>
-      <c r="M4" s="53"/>
-      <c r="N4" s="53"/>
-      <c r="O4" s="53"/>
-      <c r="P4" s="54"/>
+      <c r="I4" s="62"/>
+      <c r="J4" s="63"/>
+      <c r="K4" s="63"/>
+      <c r="L4" s="63"/>
+      <c r="M4" s="63"/>
+      <c r="N4" s="63"/>
+      <c r="O4" s="63"/>
+      <c r="P4" s="64"/>
       <c r="Q4" s="4"/>
       <c r="R4" s="2"/>
     </row>
     <row r="5" spans="1:20" s="1" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="67" t="s">
+      <c r="A5" s="60" t="s">
         <v>369</v>
       </c>
-      <c r="B5" s="68"/>
-      <c r="C5" s="68"/>
-      <c r="D5" s="66" t="s">
-        <v>688</v>
-      </c>
-      <c r="E5" s="66"/>
-      <c r="F5" s="66"/>
-      <c r="G5" s="66"/>
+      <c r="B5" s="61"/>
+      <c r="C5" s="61"/>
+      <c r="D5" s="59"/>
+      <c r="E5" s="59"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="59"/>
       <c r="H5" s="3" t="s">
         <v>370</v>
       </c>
-      <c r="I5" s="52"/>
-      <c r="J5" s="53"/>
-      <c r="K5" s="53"/>
-      <c r="L5" s="53"/>
-      <c r="M5" s="53"/>
-      <c r="N5" s="53"/>
-      <c r="O5" s="53"/>
-      <c r="P5" s="54"/>
+      <c r="I5" s="62"/>
+      <c r="J5" s="63"/>
+      <c r="K5" s="63"/>
+      <c r="L5" s="63"/>
+      <c r="M5" s="63"/>
+      <c r="N5" s="63"/>
+      <c r="O5" s="63"/>
+      <c r="P5" s="64"/>
       <c r="Q5" s="4"/>
       <c r="R5" s="2"/>
     </row>
     <row r="6" spans="1:20" s="1" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="69" t="s">
+      <c r="A6" s="56" t="s">
         <v>679</v>
       </c>
-      <c r="B6" s="70"/>
-      <c r="C6" s="71"/>
-      <c r="D6" s="66" t="s">
-        <v>688</v>
-      </c>
-      <c r="E6" s="66"/>
-      <c r="F6" s="66"/>
-      <c r="G6" s="66"/>
+      <c r="B6" s="57"/>
+      <c r="C6" s="58"/>
+      <c r="D6" s="59"/>
+      <c r="E6" s="59"/>
+      <c r="F6" s="59"/>
+      <c r="G6" s="59"/>
       <c r="H6" s="3" t="s">
         <v>372</v>
       </c>
-      <c r="I6" s="52"/>
-      <c r="J6" s="53"/>
-      <c r="K6" s="53"/>
-      <c r="L6" s="53"/>
-      <c r="M6" s="53"/>
-      <c r="N6" s="53"/>
-      <c r="O6" s="53"/>
-      <c r="P6" s="54"/>
+      <c r="I6" s="62"/>
+      <c r="J6" s="63"/>
+      <c r="K6" s="63"/>
+      <c r="L6" s="63"/>
+      <c r="M6" s="63"/>
+      <c r="N6" s="63"/>
+      <c r="O6" s="63"/>
+      <c r="P6" s="64"/>
       <c r="Q6" s="4"/>
       <c r="R6" s="2"/>
     </row>
     <row r="7" spans="1:20" s="1" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="69" t="s">
+      <c r="A7" s="56" t="s">
         <v>680</v>
       </c>
-      <c r="B7" s="70"/>
-      <c r="C7" s="71"/>
-      <c r="D7" s="66" t="s">
-        <v>688</v>
-      </c>
-      <c r="E7" s="66"/>
-      <c r="F7" s="66"/>
-      <c r="G7" s="66"/>
+      <c r="B7" s="57"/>
+      <c r="C7" s="58"/>
+      <c r="D7" s="59"/>
+      <c r="E7" s="59"/>
+      <c r="F7" s="59"/>
+      <c r="G7" s="59"/>
       <c r="H7" s="3" t="s">
         <v>373</v>
       </c>
-      <c r="I7" s="52"/>
-      <c r="J7" s="53"/>
-      <c r="K7" s="53"/>
-      <c r="L7" s="53"/>
-      <c r="M7" s="53"/>
-      <c r="N7" s="53"/>
-      <c r="O7" s="53"/>
-      <c r="P7" s="54"/>
+      <c r="I7" s="62"/>
+      <c r="J7" s="63"/>
+      <c r="K7" s="63"/>
+      <c r="L7" s="63"/>
+      <c r="M7" s="63"/>
+      <c r="N7" s="63"/>
+      <c r="O7" s="63"/>
+      <c r="P7" s="64"/>
       <c r="Q7" s="4"/>
       <c r="R7" s="2"/>
     </row>
     <row r="8" spans="1:20" s="1" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="69" t="s">
+      <c r="A8" s="56" t="s">
         <v>687</v>
       </c>
-      <c r="B8" s="70"/>
-      <c r="C8" s="71"/>
-      <c r="D8" s="66" t="s">
-        <v>688</v>
-      </c>
-      <c r="E8" s="66"/>
-      <c r="F8" s="66"/>
-      <c r="G8" s="66"/>
-      <c r="H8" s="72" t="s">
+      <c r="B8" s="57"/>
+      <c r="C8" s="58"/>
+      <c r="D8" s="59"/>
+      <c r="E8" s="59"/>
+      <c r="F8" s="59"/>
+      <c r="G8" s="59"/>
+      <c r="H8" s="71" t="s">
         <v>375</v>
       </c>
-      <c r="I8" s="75"/>
-      <c r="J8" s="76"/>
-      <c r="K8" s="76"/>
-      <c r="L8" s="76"/>
-      <c r="M8" s="76"/>
-      <c r="N8" s="76"/>
-      <c r="O8" s="76"/>
-      <c r="P8" s="77"/>
+      <c r="I8" s="74"/>
+      <c r="J8" s="75"/>
+      <c r="K8" s="75"/>
+      <c r="L8" s="75"/>
+      <c r="M8" s="75"/>
+      <c r="N8" s="75"/>
+      <c r="O8" s="75"/>
+      <c r="P8" s="76"/>
       <c r="Q8" s="4"/>
       <c r="R8" s="2"/>
     </row>
     <row r="9" spans="1:20" s="1" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="67" t="s">
+      <c r="A9" s="60" t="s">
         <v>371</v>
       </c>
-      <c r="B9" s="68"/>
-      <c r="C9" s="68"/>
-      <c r="D9" s="66" t="s">
-        <v>688</v>
-      </c>
-      <c r="E9" s="66"/>
-      <c r="F9" s="66"/>
-      <c r="G9" s="66"/>
-      <c r="H9" s="73"/>
-      <c r="I9" s="78"/>
-      <c r="J9" s="79"/>
-      <c r="K9" s="79"/>
-      <c r="L9" s="79"/>
-      <c r="M9" s="79"/>
-      <c r="N9" s="79"/>
-      <c r="O9" s="79"/>
-      <c r="P9" s="80"/>
+      <c r="B9" s="61"/>
+      <c r="C9" s="61"/>
+      <c r="D9" s="59"/>
+      <c r="E9" s="59"/>
+      <c r="F9" s="59"/>
+      <c r="G9" s="59"/>
+      <c r="H9" s="72"/>
+      <c r="I9" s="77"/>
+      <c r="J9" s="78"/>
+      <c r="K9" s="78"/>
+      <c r="L9" s="78"/>
+      <c r="M9" s="78"/>
+      <c r="N9" s="78"/>
+      <c r="O9" s="78"/>
+      <c r="P9" s="79"/>
       <c r="Q9" s="4"/>
       <c r="R9" s="2"/>
     </row>
     <row r="10" spans="1:20" s="1" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="69" t="s">
-        <v>695</v>
-      </c>
-      <c r="B10" s="70"/>
-      <c r="C10" s="71"/>
-      <c r="D10" s="66" t="s">
-        <v>688</v>
-      </c>
-      <c r="E10" s="66"/>
-      <c r="F10" s="66"/>
-      <c r="G10" s="66"/>
-      <c r="H10" s="73"/>
-      <c r="I10" s="78"/>
-      <c r="J10" s="79"/>
-      <c r="K10" s="79"/>
-      <c r="L10" s="79"/>
-      <c r="M10" s="79"/>
-      <c r="N10" s="79"/>
-      <c r="O10" s="79"/>
-      <c r="P10" s="80"/>
+      <c r="A10" s="56" t="s">
+        <v>694</v>
+      </c>
+      <c r="B10" s="57"/>
+      <c r="C10" s="58"/>
+      <c r="D10" s="59"/>
+      <c r="E10" s="59"/>
+      <c r="F10" s="59"/>
+      <c r="G10" s="59"/>
+      <c r="H10" s="72"/>
+      <c r="I10" s="77"/>
+      <c r="J10" s="78"/>
+      <c r="K10" s="78"/>
+      <c r="L10" s="78"/>
+      <c r="M10" s="78"/>
+      <c r="N10" s="78"/>
+      <c r="O10" s="78"/>
+      <c r="P10" s="79"/>
       <c r="Q10" s="4"/>
       <c r="R10" s="2"/>
     </row>
     <row r="11" spans="1:20" s="1" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="67" t="s">
-        <v>689</v>
-      </c>
-      <c r="B11" s="68"/>
-      <c r="C11" s="68"/>
-      <c r="D11" s="66" t="s">
+      <c r="A11" s="60" t="s">
         <v>688</v>
       </c>
-      <c r="E11" s="66"/>
-      <c r="F11" s="66"/>
-      <c r="G11" s="66"/>
-      <c r="H11" s="73"/>
-      <c r="I11" s="78"/>
-      <c r="J11" s="79"/>
-      <c r="K11" s="79"/>
-      <c r="L11" s="79"/>
-      <c r="M11" s="79"/>
-      <c r="N11" s="79"/>
-      <c r="O11" s="79"/>
-      <c r="P11" s="80"/>
+      <c r="B11" s="61"/>
+      <c r="C11" s="61"/>
+      <c r="D11" s="59"/>
+      <c r="E11" s="59"/>
+      <c r="F11" s="59"/>
+      <c r="G11" s="59"/>
+      <c r="H11" s="72"/>
+      <c r="I11" s="77"/>
+      <c r="J11" s="78"/>
+      <c r="K11" s="78"/>
+      <c r="L11" s="78"/>
+      <c r="M11" s="78"/>
+      <c r="N11" s="78"/>
+      <c r="O11" s="78"/>
+      <c r="P11" s="79"/>
       <c r="Q11" s="4"/>
       <c r="R11" s="2"/>
     </row>
     <row r="12" spans="1:20" s="1" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="69" t="s">
+      <c r="A12" s="56" t="s">
         <v>681</v>
       </c>
-      <c r="B12" s="70"/>
-      <c r="C12" s="71"/>
-      <c r="D12" s="66" t="s">
-        <v>688</v>
-      </c>
-      <c r="E12" s="66"/>
-      <c r="F12" s="66"/>
-      <c r="G12" s="66"/>
-      <c r="H12" s="74"/>
-      <c r="I12" s="81"/>
-      <c r="J12" s="82"/>
-      <c r="K12" s="82"/>
-      <c r="L12" s="82"/>
-      <c r="M12" s="82"/>
-      <c r="N12" s="82"/>
-      <c r="O12" s="82"/>
-      <c r="P12" s="83"/>
+      <c r="B12" s="57"/>
+      <c r="C12" s="58"/>
+      <c r="D12" s="59"/>
+      <c r="E12" s="59"/>
+      <c r="F12" s="59"/>
+      <c r="G12" s="59"/>
+      <c r="H12" s="73"/>
+      <c r="I12" s="80"/>
+      <c r="J12" s="81"/>
+      <c r="K12" s="81"/>
+      <c r="L12" s="81"/>
+      <c r="M12" s="81"/>
+      <c r="N12" s="81"/>
+      <c r="O12" s="81"/>
+      <c r="P12" s="82"/>
       <c r="Q12" s="4"/>
       <c r="R12" s="2"/>
     </row>
     <row r="13" spans="1:20" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="86" t="s">
+      <c r="A13" s="55" t="s">
         <v>374</v>
       </c>
-      <c r="B13" s="85"/>
-      <c r="C13" s="85"/>
-      <c r="D13" s="85"/>
-      <c r="E13" s="85"/>
-      <c r="F13" s="85"/>
-      <c r="G13" s="85"/>
-      <c r="H13" s="85"/>
-      <c r="I13" s="85"/>
-      <c r="J13" s="85"/>
-      <c r="K13" s="85"/>
-      <c r="L13" s="85"/>
-      <c r="M13" s="85"/>
-      <c r="N13" s="85"/>
-      <c r="O13" s="85"/>
-      <c r="P13" s="85"/>
+      <c r="B13" s="54"/>
+      <c r="C13" s="54"/>
+      <c r="D13" s="54"/>
+      <c r="E13" s="54"/>
+      <c r="F13" s="54"/>
+      <c r="G13" s="54"/>
+      <c r="H13" s="54"/>
+      <c r="I13" s="54"/>
+      <c r="J13" s="54"/>
+      <c r="K13" s="54"/>
+      <c r="L13" s="54"/>
+      <c r="M13" s="54"/>
+      <c r="N13" s="54"/>
+      <c r="O13" s="54"/>
+      <c r="P13" s="54"/>
       <c r="R13" s="2"/>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.25">
@@ -3614,10 +3566,10 @@
         <v>366</v>
       </c>
       <c r="Q15" s="49" t="s">
+        <v>690</v>
+      </c>
+      <c r="R15" s="49" t="s">
         <v>691</v>
-      </c>
-      <c r="R15" s="49" t="s">
-        <v>692</v>
       </c>
       <c r="S15" s="6"/>
       <c r="T15" s="6"/>
@@ -9525,8 +9477,8 @@
       <c r="H114" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I114" s="36">
-        <v>43.6</v>
+      <c r="I114" s="27">
+        <v>10.9</v>
       </c>
       <c r="J114" s="25" t="s">
         <v>377</v>
@@ -9542,11 +9494,11 @@
       </c>
       <c r="N114" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O114" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P114" s="8"/>
       <c r="Q114" s="50">
@@ -9583,8 +9535,8 @@
       <c r="H115" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I115" s="36">
-        <v>43.6</v>
+      <c r="I115" s="27">
+        <v>10.9</v>
       </c>
       <c r="J115" s="25" t="s">
         <v>377</v>
@@ -9600,11 +9552,11 @@
       </c>
       <c r="N115" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O115" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P115" s="8"/>
       <c r="Q115" s="50">
@@ -9641,8 +9593,8 @@
       <c r="H116" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I116" s="36">
-        <v>43.6</v>
+      <c r="I116" s="27">
+        <v>10.9</v>
       </c>
       <c r="J116" s="25" t="s">
         <v>377</v>
@@ -9658,11 +9610,11 @@
       </c>
       <c r="N116" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O116" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P116" s="8"/>
       <c r="Q116" s="50">
@@ -9699,8 +9651,8 @@
       <c r="H117" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I117" s="36">
-        <v>43.6</v>
+      <c r="I117" s="27">
+        <v>10.9</v>
       </c>
       <c r="J117" s="25" t="s">
         <v>377</v>
@@ -9716,11 +9668,11 @@
       </c>
       <c r="N117" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O117" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P117" s="8"/>
       <c r="Q117" s="50">
@@ -9757,8 +9709,8 @@
       <c r="H118" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I118" s="36">
-        <v>43.6</v>
+      <c r="I118" s="27">
+        <v>10.9</v>
       </c>
       <c r="J118" s="25" t="s">
         <v>377</v>
@@ -9774,11 +9726,11 @@
       </c>
       <c r="N118" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O118" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P118" s="8"/>
       <c r="Q118" s="50">
@@ -9815,8 +9767,8 @@
       <c r="H119" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I119" s="36">
-        <v>43.6</v>
+      <c r="I119" s="27">
+        <v>10.9</v>
       </c>
       <c r="J119" s="25" t="s">
         <v>377</v>
@@ -9832,11 +9784,11 @@
       </c>
       <c r="N119" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O119" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P119" s="8"/>
       <c r="Q119" s="50">
@@ -9873,8 +9825,8 @@
       <c r="H120" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I120" s="36">
-        <v>43.6</v>
+      <c r="I120" s="27">
+        <v>10.9</v>
       </c>
       <c r="J120" s="25" t="s">
         <v>377</v>
@@ -9890,11 +9842,11 @@
       </c>
       <c r="N120" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O120" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P120" s="8"/>
       <c r="Q120" s="50">
@@ -9931,8 +9883,8 @@
       <c r="H121" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I121" s="36">
-        <v>43.6</v>
+      <c r="I121" s="27">
+        <v>10.9</v>
       </c>
       <c r="J121" s="25" t="s">
         <v>377</v>
@@ -9948,11 +9900,11 @@
       </c>
       <c r="N121" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O121" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P121" s="8"/>
       <c r="Q121" s="50">
@@ -9989,8 +9941,8 @@
       <c r="H122" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I122" s="36">
-        <v>43.6</v>
+      <c r="I122" s="27">
+        <v>10.9</v>
       </c>
       <c r="J122" s="25" t="s">
         <v>377</v>
@@ -10006,11 +9958,11 @@
       </c>
       <c r="N122" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O122" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P122" s="8"/>
       <c r="Q122" s="50">
@@ -10047,8 +9999,8 @@
       <c r="H123" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I123" s="36">
-        <v>43.6</v>
+      <c r="I123" s="27">
+        <v>10.9</v>
       </c>
       <c r="J123" s="25" t="s">
         <v>377</v>
@@ -10064,11 +10016,11 @@
       </c>
       <c r="N123" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O123" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P123" s="8"/>
       <c r="Q123" s="50">
@@ -10105,8 +10057,8 @@
       <c r="H124" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I124" s="36">
-        <v>43.6</v>
+      <c r="I124" s="27">
+        <v>10.9</v>
       </c>
       <c r="J124" s="25" t="s">
         <v>377</v>
@@ -10122,11 +10074,11 @@
       </c>
       <c r="N124" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O124" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P124" s="8"/>
       <c r="Q124" s="50">
@@ -10163,8 +10115,8 @@
       <c r="H125" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I125" s="36">
-        <v>43.6</v>
+      <c r="I125" s="27">
+        <v>10.9</v>
       </c>
       <c r="J125" s="25" t="s">
         <v>377</v>
@@ -10180,11 +10132,11 @@
       </c>
       <c r="N125" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O125" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P125" s="8"/>
       <c r="Q125" s="50">
@@ -10221,8 +10173,8 @@
       <c r="H126" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I126" s="36">
-        <v>43.6</v>
+      <c r="I126" s="27">
+        <v>10.9</v>
       </c>
       <c r="J126" s="25" t="s">
         <v>377</v>
@@ -10238,11 +10190,11 @@
       </c>
       <c r="N126" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O126" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P126" s="8"/>
       <c r="Q126" s="50">
@@ -10279,8 +10231,8 @@
       <c r="H127" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I127" s="36">
-        <v>43.6</v>
+      <c r="I127" s="27">
+        <v>10.9</v>
       </c>
       <c r="J127" s="25" t="s">
         <v>377</v>
@@ -10296,11 +10248,11 @@
       </c>
       <c r="N127" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O127" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P127" s="8"/>
       <c r="Q127" s="50">
@@ -10337,8 +10289,8 @@
       <c r="H128" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I128" s="36">
-        <v>43.6</v>
+      <c r="I128" s="27">
+        <v>10.9</v>
       </c>
       <c r="J128" s="25" t="s">
         <v>377</v>
@@ -10354,11 +10306,11 @@
       </c>
       <c r="N128" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O128" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P128" s="8"/>
       <c r="Q128" s="50">
@@ -10395,8 +10347,8 @@
       <c r="H129" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I129" s="36">
-        <v>43.6</v>
+      <c r="I129" s="27">
+        <v>10.9</v>
       </c>
       <c r="J129" s="25" t="s">
         <v>377</v>
@@ -10412,11 +10364,11 @@
       </c>
       <c r="N129" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O129" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P129" s="8"/>
       <c r="Q129" s="50">
@@ -10453,8 +10405,8 @@
       <c r="H130" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I130" s="36">
-        <v>43.6</v>
+      <c r="I130" s="27">
+        <v>10.9</v>
       </c>
       <c r="J130" s="25" t="s">
         <v>377</v>
@@ -10470,11 +10422,11 @@
       </c>
       <c r="N130" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O130" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P130" s="8"/>
       <c r="Q130" s="50">
@@ -10511,8 +10463,8 @@
       <c r="H131" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I131" s="36">
-        <v>43.6</v>
+      <c r="I131" s="27">
+        <v>10.9</v>
       </c>
       <c r="J131" s="25" t="s">
         <v>377</v>
@@ -10528,11 +10480,11 @@
       </c>
       <c r="N131" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O131" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P131" s="8"/>
       <c r="Q131" s="50">
@@ -10569,8 +10521,8 @@
       <c r="H132" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I132" s="36">
-        <v>43.6</v>
+      <c r="I132" s="27">
+        <v>10.9</v>
       </c>
       <c r="J132" s="25" t="s">
         <v>377</v>
@@ -10586,11 +10538,11 @@
       </c>
       <c r="N132" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O132" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P132" s="8"/>
       <c r="Q132" s="50">
@@ -10627,8 +10579,8 @@
       <c r="H133" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I133" s="36">
-        <v>43.6</v>
+      <c r="I133" s="27">
+        <v>10.9</v>
       </c>
       <c r="J133" s="25" t="s">
         <v>377</v>
@@ -10644,11 +10596,11 @@
       </c>
       <c r="N133" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O133" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P133" s="8"/>
       <c r="Q133" s="50">
@@ -10685,8 +10637,8 @@
       <c r="H134" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I134" s="36">
-        <v>43.6</v>
+      <c r="I134" s="27">
+        <v>10.9</v>
       </c>
       <c r="J134" s="25" t="s">
         <v>377</v>
@@ -10702,11 +10654,11 @@
       </c>
       <c r="N134" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O134" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P134" s="8"/>
       <c r="Q134" s="50">
@@ -10743,8 +10695,8 @@
       <c r="H135" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I135" s="36">
-        <v>43.6</v>
+      <c r="I135" s="27">
+        <v>10.9</v>
       </c>
       <c r="J135" s="25" t="s">
         <v>377</v>
@@ -10760,11 +10712,11 @@
       </c>
       <c r="N135" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O135" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P135" s="8"/>
       <c r="Q135" s="50">
@@ -10801,8 +10753,8 @@
       <c r="H136" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I136" s="36">
-        <v>43.6</v>
+      <c r="I136" s="27">
+        <v>10.9</v>
       </c>
       <c r="J136" s="25" t="s">
         <v>377</v>
@@ -10818,11 +10770,11 @@
       </c>
       <c r="N136" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O136" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P136" s="8"/>
       <c r="Q136" s="50">
@@ -10859,8 +10811,8 @@
       <c r="H137" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I137" s="36">
-        <v>43.6</v>
+      <c r="I137" s="27">
+        <v>10.9</v>
       </c>
       <c r="J137" s="25" t="s">
         <v>377</v>
@@ -10876,11 +10828,11 @@
       </c>
       <c r="N137" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O137" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P137" s="8"/>
       <c r="Q137" s="50">
@@ -10975,8 +10927,8 @@
       <c r="H139" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I139" s="36">
-        <v>43.6</v>
+      <c r="I139" s="27">
+        <v>10.9</v>
       </c>
       <c r="J139" s="25" t="s">
         <v>377</v>
@@ -10992,11 +10944,11 @@
       </c>
       <c r="N139" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O139" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P139" s="8"/>
       <c r="Q139" s="50">
@@ -11033,8 +10985,8 @@
       <c r="H140" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I140" s="36">
-        <v>43.6</v>
+      <c r="I140" s="27">
+        <v>10.9</v>
       </c>
       <c r="J140" s="25" t="s">
         <v>377</v>
@@ -11050,11 +11002,11 @@
       </c>
       <c r="N140" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O140" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P140" s="8"/>
       <c r="Q140" s="50">
@@ -11091,8 +11043,8 @@
       <c r="H141" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I141" s="36">
-        <v>43.6</v>
+      <c r="I141" s="27">
+        <v>10.9</v>
       </c>
       <c r="J141" s="25" t="s">
         <v>377</v>
@@ -11108,11 +11060,11 @@
       </c>
       <c r="N141" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O141" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P141" s="8"/>
       <c r="Q141" s="50">
@@ -11149,8 +11101,8 @@
       <c r="H142" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I142" s="36">
-        <v>43.6</v>
+      <c r="I142" s="27">
+        <v>10.9</v>
       </c>
       <c r="J142" s="25" t="s">
         <v>377</v>
@@ -11166,11 +11118,11 @@
       </c>
       <c r="N142" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O142" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P142" s="8"/>
       <c r="Q142" s="50">
@@ -11207,8 +11159,8 @@
       <c r="H143" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I143" s="36">
-        <v>43.6</v>
+      <c r="I143" s="27">
+        <v>10.9</v>
       </c>
       <c r="J143" s="25" t="s">
         <v>377</v>
@@ -11224,11 +11176,11 @@
       </c>
       <c r="N143" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O143" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P143" s="8"/>
       <c r="Q143" s="50">
@@ -11265,8 +11217,8 @@
       <c r="H144" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I144" s="36">
-        <v>43.6</v>
+      <c r="I144" s="27">
+        <v>10.9</v>
       </c>
       <c r="J144" s="25" t="s">
         <v>377</v>
@@ -11282,11 +11234,11 @@
       </c>
       <c r="N144" s="30">
         <f t="shared" si="4"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O144" s="30">
         <f t="shared" si="5"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P144" s="8"/>
       <c r="Q144" s="50">
@@ -11323,8 +11275,8 @@
       <c r="H145" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I145" s="36">
-        <v>43.6</v>
+      <c r="I145" s="27">
+        <v>10.9</v>
       </c>
       <c r="J145" s="25" t="s">
         <v>377</v>
@@ -11340,11 +11292,11 @@
       </c>
       <c r="N145" s="30">
         <f t="shared" ref="N145:N208" si="8">I145*(1-M145)</f>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O145" s="30">
         <f t="shared" ref="O145:O208" si="9">N145*(1+J145)</f>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P145" s="8"/>
       <c r="Q145" s="50">
@@ -11381,8 +11333,8 @@
       <c r="H146" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I146" s="36">
-        <v>43.6</v>
+      <c r="I146" s="27">
+        <v>10.9</v>
       </c>
       <c r="J146" s="25" t="s">
         <v>377</v>
@@ -11398,11 +11350,11 @@
       </c>
       <c r="N146" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O146" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P146" s="8"/>
       <c r="Q146" s="50">
@@ -11439,8 +11391,8 @@
       <c r="H147" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I147" s="36">
-        <v>43.6</v>
+      <c r="I147" s="27">
+        <v>10.9</v>
       </c>
       <c r="J147" s="25" t="s">
         <v>377</v>
@@ -11456,11 +11408,11 @@
       </c>
       <c r="N147" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O147" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P147" s="8"/>
       <c r="Q147" s="50">
@@ -11497,8 +11449,8 @@
       <c r="H148" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I148" s="36">
-        <v>43.6</v>
+      <c r="I148" s="27">
+        <v>10.9</v>
       </c>
       <c r="J148" s="25" t="s">
         <v>377</v>
@@ -11514,11 +11466,11 @@
       </c>
       <c r="N148" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O148" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P148" s="8"/>
       <c r="Q148" s="50">
@@ -11555,8 +11507,8 @@
       <c r="H149" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I149" s="36">
-        <v>43.6</v>
+      <c r="I149" s="27">
+        <v>10.9</v>
       </c>
       <c r="J149" s="25" t="s">
         <v>377</v>
@@ -11572,11 +11524,11 @@
       </c>
       <c r="N149" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O149" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P149" s="8"/>
       <c r="Q149" s="50">
@@ -11613,8 +11565,8 @@
       <c r="H150" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I150" s="36">
-        <v>43.6</v>
+      <c r="I150" s="27">
+        <v>10.9</v>
       </c>
       <c r="J150" s="25" t="s">
         <v>377</v>
@@ -11630,11 +11582,11 @@
       </c>
       <c r="N150" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O150" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P150" s="8"/>
       <c r="Q150" s="50">
@@ -11671,8 +11623,8 @@
       <c r="H151" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I151" s="36">
-        <v>43.6</v>
+      <c r="I151" s="27">
+        <v>10.9</v>
       </c>
       <c r="J151" s="25" t="s">
         <v>377</v>
@@ -11688,11 +11640,11 @@
       </c>
       <c r="N151" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O151" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P151" s="8"/>
       <c r="Q151" s="50">
@@ -11729,8 +11681,8 @@
       <c r="H152" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I152" s="36">
-        <v>43.6</v>
+      <c r="I152" s="27">
+        <v>10.9</v>
       </c>
       <c r="J152" s="25" t="s">
         <v>377</v>
@@ -11746,11 +11698,11 @@
       </c>
       <c r="N152" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O152" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P152" s="8"/>
       <c r="Q152" s="50">
@@ -11787,8 +11739,8 @@
       <c r="H153" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I153" s="36">
-        <v>43.6</v>
+      <c r="I153" s="27">
+        <v>10.9</v>
       </c>
       <c r="J153" s="25" t="s">
         <v>377</v>
@@ -11804,11 +11756,11 @@
       </c>
       <c r="N153" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O153" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P153" s="8"/>
       <c r="Q153" s="50">
@@ -11845,8 +11797,8 @@
       <c r="H154" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I154" s="36">
-        <v>43.6</v>
+      <c r="I154" s="27">
+        <v>10.9</v>
       </c>
       <c r="J154" s="25" t="s">
         <v>377</v>
@@ -11862,11 +11814,11 @@
       </c>
       <c r="N154" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O154" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P154" s="8"/>
       <c r="Q154" s="50">
@@ -11903,8 +11855,8 @@
       <c r="H155" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I155" s="36">
-        <v>43.6</v>
+      <c r="I155" s="27">
+        <v>10.9</v>
       </c>
       <c r="J155" s="25" t="s">
         <v>377</v>
@@ -11920,11 +11872,11 @@
       </c>
       <c r="N155" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O155" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P155" s="8"/>
       <c r="Q155" s="50">
@@ -11961,8 +11913,8 @@
       <c r="H156" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I156" s="36">
-        <v>43.6</v>
+      <c r="I156" s="27">
+        <v>10.9</v>
       </c>
       <c r="J156" s="25" t="s">
         <v>377</v>
@@ -11978,11 +11930,11 @@
       </c>
       <c r="N156" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O156" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P156" s="8"/>
       <c r="Q156" s="50">
@@ -12019,8 +11971,8 @@
       <c r="H157" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I157" s="36">
-        <v>43.6</v>
+      <c r="I157" s="27">
+        <v>10.9</v>
       </c>
       <c r="J157" s="25" t="s">
         <v>377</v>
@@ -12036,11 +11988,11 @@
       </c>
       <c r="N157" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O157" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P157" s="8"/>
       <c r="Q157" s="50">
@@ -12077,8 +12029,8 @@
       <c r="H158" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I158" s="36">
-        <v>43.6</v>
+      <c r="I158" s="27">
+        <v>10.9</v>
       </c>
       <c r="J158" s="25" t="s">
         <v>377</v>
@@ -12094,11 +12046,11 @@
       </c>
       <c r="N158" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O158" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P158" s="8"/>
       <c r="Q158" s="50">
@@ -12135,8 +12087,8 @@
       <c r="H159" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I159" s="36">
-        <v>43.6</v>
+      <c r="I159" s="27">
+        <v>10.9</v>
       </c>
       <c r="J159" s="25" t="s">
         <v>377</v>
@@ -12152,11 +12104,11 @@
       </c>
       <c r="N159" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O159" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P159" s="8"/>
       <c r="Q159" s="50">
@@ -12193,8 +12145,8 @@
       <c r="H160" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I160" s="36">
-        <v>43.6</v>
+      <c r="I160" s="27">
+        <v>10.9</v>
       </c>
       <c r="J160" s="25" t="s">
         <v>377</v>
@@ -12210,11 +12162,11 @@
       </c>
       <c r="N160" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O160" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P160" s="8"/>
       <c r="Q160" s="50">
@@ -12251,8 +12203,8 @@
       <c r="H161" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I161" s="36">
-        <v>43.6</v>
+      <c r="I161" s="27">
+        <v>10.9</v>
       </c>
       <c r="J161" s="25" t="s">
         <v>377</v>
@@ -12268,11 +12220,11 @@
       </c>
       <c r="N161" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O161" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P161" s="8"/>
       <c r="Q161" s="50">
@@ -12309,8 +12261,8 @@
       <c r="H162" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I162" s="36">
-        <v>43.6</v>
+      <c r="I162" s="27">
+        <v>10.9</v>
       </c>
       <c r="J162" s="25" t="s">
         <v>377</v>
@@ -12326,11 +12278,11 @@
       </c>
       <c r="N162" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O162" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P162" s="8"/>
       <c r="Q162" s="50">
@@ -12425,8 +12377,8 @@
       <c r="H164" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I164" s="36">
-        <v>43.6</v>
+      <c r="I164" s="27">
+        <v>10.9</v>
       </c>
       <c r="J164" s="25" t="s">
         <v>377</v>
@@ -12442,11 +12394,11 @@
       </c>
       <c r="N164" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O164" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P164" s="8"/>
       <c r="Q164" s="50">
@@ -12483,8 +12435,8 @@
       <c r="H165" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I165" s="36">
-        <v>43.6</v>
+      <c r="I165" s="27">
+        <v>10.9</v>
       </c>
       <c r="J165" s="25" t="s">
         <v>377</v>
@@ -12500,11 +12452,11 @@
       </c>
       <c r="N165" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O165" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P165" s="8"/>
       <c r="Q165" s="50">
@@ -12541,8 +12493,8 @@
       <c r="H166" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I166" s="36">
-        <v>43.6</v>
+      <c r="I166" s="27">
+        <v>10.9</v>
       </c>
       <c r="J166" s="25" t="s">
         <v>377</v>
@@ -12558,11 +12510,11 @@
       </c>
       <c r="N166" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O166" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P166" s="8"/>
       <c r="Q166" s="50">
@@ -12599,8 +12551,8 @@
       <c r="H167" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I167" s="36">
-        <v>43.6</v>
+      <c r="I167" s="27">
+        <v>10.9</v>
       </c>
       <c r="J167" s="25" t="s">
         <v>377</v>
@@ -12616,11 +12568,11 @@
       </c>
       <c r="N167" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O167" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P167" s="8"/>
       <c r="Q167" s="50">
@@ -12657,8 +12609,8 @@
       <c r="H168" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I168" s="36">
-        <v>43.6</v>
+      <c r="I168" s="27">
+        <v>10.9</v>
       </c>
       <c r="J168" s="25" t="s">
         <v>377</v>
@@ -12674,11 +12626,11 @@
       </c>
       <c r="N168" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O168" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P168" s="8"/>
       <c r="Q168" s="50">
@@ -12715,8 +12667,8 @@
       <c r="H169" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I169" s="36">
-        <v>43.6</v>
+      <c r="I169" s="27">
+        <v>10.9</v>
       </c>
       <c r="J169" s="25" t="s">
         <v>377</v>
@@ -12732,11 +12684,11 @@
       </c>
       <c r="N169" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O169" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P169" s="8"/>
       <c r="Q169" s="50">
@@ -12831,8 +12783,8 @@
       <c r="H171" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I171" s="36">
-        <v>43.6</v>
+      <c r="I171" s="27">
+        <v>10.9</v>
       </c>
       <c r="J171" s="25" t="s">
         <v>377</v>
@@ -12848,11 +12800,11 @@
       </c>
       <c r="N171" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O171" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P171" s="8"/>
       <c r="Q171" s="50">
@@ -12889,8 +12841,8 @@
       <c r="H172" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I172" s="36">
-        <v>43.6</v>
+      <c r="I172" s="27">
+        <v>10.9</v>
       </c>
       <c r="J172" s="25" t="s">
         <v>377</v>
@@ -12906,11 +12858,11 @@
       </c>
       <c r="N172" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O172" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P172" s="8"/>
       <c r="Q172" s="50">
@@ -12947,8 +12899,8 @@
       <c r="H173" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I173" s="36">
-        <v>43.6</v>
+      <c r="I173" s="27">
+        <v>10.9</v>
       </c>
       <c r="J173" s="25" t="s">
         <v>377</v>
@@ -12964,11 +12916,11 @@
       </c>
       <c r="N173" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O173" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P173" s="8"/>
       <c r="Q173" s="50">
@@ -13005,8 +12957,8 @@
       <c r="H174" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I174" s="36">
-        <v>43.6</v>
+      <c r="I174" s="27">
+        <v>10.9</v>
       </c>
       <c r="J174" s="25" t="s">
         <v>377</v>
@@ -13022,11 +12974,11 @@
       </c>
       <c r="N174" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O174" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P174" s="8"/>
       <c r="Q174" s="50">
@@ -13063,8 +13015,8 @@
       <c r="H175" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I175" s="36">
-        <v>43.6</v>
+      <c r="I175" s="27">
+        <v>10.9</v>
       </c>
       <c r="J175" s="25" t="s">
         <v>377</v>
@@ -13080,11 +13032,11 @@
       </c>
       <c r="N175" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O175" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P175" s="8"/>
       <c r="Q175" s="50">
@@ -13121,8 +13073,8 @@
       <c r="H176" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I176" s="36">
-        <v>43.6</v>
+      <c r="I176" s="27">
+        <v>10.9</v>
       </c>
       <c r="J176" s="25" t="s">
         <v>377</v>
@@ -13138,11 +13090,11 @@
       </c>
       <c r="N176" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O176" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P176" s="8"/>
       <c r="Q176" s="50">
@@ -13237,8 +13189,8 @@
       <c r="H178" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I178" s="36">
-        <v>43.6</v>
+      <c r="I178" s="27">
+        <v>10.9</v>
       </c>
       <c r="J178" s="25" t="s">
         <v>377</v>
@@ -13254,11 +13206,11 @@
       </c>
       <c r="N178" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O178" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P178" s="8"/>
       <c r="Q178" s="50">
@@ -13295,8 +13247,8 @@
       <c r="H179" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I179" s="36">
-        <v>43.6</v>
+      <c r="I179" s="27">
+        <v>10.9</v>
       </c>
       <c r="J179" s="25" t="s">
         <v>377</v>
@@ -13312,11 +13264,11 @@
       </c>
       <c r="N179" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O179" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P179" s="8"/>
       <c r="Q179" s="50">
@@ -13353,8 +13305,8 @@
       <c r="H180" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I180" s="36">
-        <v>43.6</v>
+      <c r="I180" s="27">
+        <v>10.9</v>
       </c>
       <c r="J180" s="25" t="s">
         <v>377</v>
@@ -13370,11 +13322,11 @@
       </c>
       <c r="N180" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O180" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P180" s="8"/>
       <c r="Q180" s="50">
@@ -13411,8 +13363,8 @@
       <c r="H181" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I181" s="36">
-        <v>43.6</v>
+      <c r="I181" s="27">
+        <v>10.9</v>
       </c>
       <c r="J181" s="25" t="s">
         <v>377</v>
@@ -13428,11 +13380,11 @@
       </c>
       <c r="N181" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O181" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P181" s="8"/>
       <c r="Q181" s="50">
@@ -13469,8 +13421,8 @@
       <c r="H182" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I182" s="36">
-        <v>43.6</v>
+      <c r="I182" s="27">
+        <v>10.9</v>
       </c>
       <c r="J182" s="25" t="s">
         <v>377</v>
@@ -13486,11 +13438,11 @@
       </c>
       <c r="N182" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O182" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P182" s="8"/>
       <c r="Q182" s="50">
@@ -13527,8 +13479,8 @@
       <c r="H183" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I183" s="36">
-        <v>43.6</v>
+      <c r="I183" s="27">
+        <v>10.9</v>
       </c>
       <c r="J183" s="25" t="s">
         <v>377</v>
@@ -13544,11 +13496,11 @@
       </c>
       <c r="N183" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O183" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P183" s="8"/>
       <c r="Q183" s="50">
@@ -13643,8 +13595,8 @@
       <c r="H185" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I185" s="36">
-        <v>43.6</v>
+      <c r="I185" s="27">
+        <v>10.9</v>
       </c>
       <c r="J185" s="25" t="s">
         <v>377</v>
@@ -13660,11 +13612,11 @@
       </c>
       <c r="N185" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O185" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P185" s="8"/>
       <c r="Q185" s="50">
@@ -13701,8 +13653,8 @@
       <c r="H186" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I186" s="36">
-        <v>43.6</v>
+      <c r="I186" s="27">
+        <v>10.9</v>
       </c>
       <c r="J186" s="25" t="s">
         <v>377</v>
@@ -13718,11 +13670,11 @@
       </c>
       <c r="N186" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O186" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P186" s="8"/>
       <c r="Q186" s="50">
@@ -13759,8 +13711,8 @@
       <c r="H187" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I187" s="36">
-        <v>43.6</v>
+      <c r="I187" s="27">
+        <v>10.9</v>
       </c>
       <c r="J187" s="25" t="s">
         <v>377</v>
@@ -13776,11 +13728,11 @@
       </c>
       <c r="N187" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O187" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P187" s="8"/>
       <c r="Q187" s="50">
@@ -13817,8 +13769,8 @@
       <c r="H188" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I188" s="36">
-        <v>43.6</v>
+      <c r="I188" s="27">
+        <v>10.9</v>
       </c>
       <c r="J188" s="25" t="s">
         <v>377</v>
@@ -13834,11 +13786,11 @@
       </c>
       <c r="N188" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O188" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P188" s="8"/>
       <c r="Q188" s="50">
@@ -13875,8 +13827,8 @@
       <c r="H189" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I189" s="36">
-        <v>43.6</v>
+      <c r="I189" s="27">
+        <v>10.9</v>
       </c>
       <c r="J189" s="25" t="s">
         <v>377</v>
@@ -13892,11 +13844,11 @@
       </c>
       <c r="N189" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O189" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P189" s="8"/>
       <c r="Q189" s="50">
@@ -13933,8 +13885,8 @@
       <c r="H190" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I190" s="36">
-        <v>43.6</v>
+      <c r="I190" s="27">
+        <v>10.9</v>
       </c>
       <c r="J190" s="25" t="s">
         <v>377</v>
@@ -13950,11 +13902,11 @@
       </c>
       <c r="N190" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O190" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P190" s="8"/>
       <c r="Q190" s="50">
@@ -14049,8 +14001,8 @@
       <c r="H192" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I192" s="36">
-        <v>43.6</v>
+      <c r="I192" s="27">
+        <v>10.9</v>
       </c>
       <c r="J192" s="25" t="s">
         <v>377</v>
@@ -14066,11 +14018,11 @@
       </c>
       <c r="N192" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O192" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P192" s="8"/>
       <c r="Q192" s="50">
@@ -14107,8 +14059,8 @@
       <c r="H193" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I193" s="36">
-        <v>43.6</v>
+      <c r="I193" s="27">
+        <v>10.9</v>
       </c>
       <c r="J193" s="25" t="s">
         <v>377</v>
@@ -14124,11 +14076,11 @@
       </c>
       <c r="N193" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O193" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P193" s="8"/>
       <c r="Q193" s="50">
@@ -14165,8 +14117,8 @@
       <c r="H194" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I194" s="36">
-        <v>43.6</v>
+      <c r="I194" s="27">
+        <v>10.9</v>
       </c>
       <c r="J194" s="25" t="s">
         <v>377</v>
@@ -14182,11 +14134,11 @@
       </c>
       <c r="N194" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O194" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P194" s="8"/>
       <c r="Q194" s="50">
@@ -14223,8 +14175,8 @@
       <c r="H195" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I195" s="36">
-        <v>43.6</v>
+      <c r="I195" s="27">
+        <v>10.9</v>
       </c>
       <c r="J195" s="25" t="s">
         <v>377</v>
@@ -14240,11 +14192,11 @@
       </c>
       <c r="N195" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O195" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P195" s="8"/>
       <c r="Q195" s="50">
@@ -14281,8 +14233,8 @@
       <c r="H196" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I196" s="36">
-        <v>43.6</v>
+      <c r="I196" s="27">
+        <v>10.9</v>
       </c>
       <c r="J196" s="25" t="s">
         <v>377</v>
@@ -14298,11 +14250,11 @@
       </c>
       <c r="N196" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O196" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P196" s="8"/>
       <c r="Q196" s="50">
@@ -14339,8 +14291,8 @@
       <c r="H197" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I197" s="36">
-        <v>43.6</v>
+      <c r="I197" s="27">
+        <v>10.9</v>
       </c>
       <c r="J197" s="25" t="s">
         <v>377</v>
@@ -14356,11 +14308,11 @@
       </c>
       <c r="N197" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O197" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P197" s="8"/>
       <c r="Q197" s="50">
@@ -14455,8 +14407,8 @@
       <c r="H199" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I199" s="36">
-        <v>43.6</v>
+      <c r="I199" s="27">
+        <v>10.9</v>
       </c>
       <c r="J199" s="25" t="s">
         <v>377</v>
@@ -14472,11 +14424,11 @@
       </c>
       <c r="N199" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O199" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P199" s="8"/>
       <c r="Q199" s="50">
@@ -14513,8 +14465,8 @@
       <c r="H200" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I200" s="36">
-        <v>43.6</v>
+      <c r="I200" s="27">
+        <v>10.9</v>
       </c>
       <c r="J200" s="25" t="s">
         <v>377</v>
@@ -14530,11 +14482,11 @@
       </c>
       <c r="N200" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O200" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P200" s="8"/>
       <c r="Q200" s="50">
@@ -14571,8 +14523,8 @@
       <c r="H201" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I201" s="36">
-        <v>43.6</v>
+      <c r="I201" s="27">
+        <v>10.9</v>
       </c>
       <c r="J201" s="25" t="s">
         <v>377</v>
@@ -14588,11 +14540,11 @@
       </c>
       <c r="N201" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O201" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P201" s="8"/>
       <c r="Q201" s="50">
@@ -14629,8 +14581,8 @@
       <c r="H202" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I202" s="36">
-        <v>43.6</v>
+      <c r="I202" s="27">
+        <v>10.9</v>
       </c>
       <c r="J202" s="25" t="s">
         <v>377</v>
@@ -14646,11 +14598,11 @@
       </c>
       <c r="N202" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O202" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P202" s="8"/>
       <c r="Q202" s="50">
@@ -14687,8 +14639,8 @@
       <c r="H203" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I203" s="36">
-        <v>43.6</v>
+      <c r="I203" s="27">
+        <v>10.9</v>
       </c>
       <c r="J203" s="25" t="s">
         <v>377</v>
@@ -14704,11 +14656,11 @@
       </c>
       <c r="N203" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O203" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P203" s="8"/>
       <c r="Q203" s="50">
@@ -14745,8 +14697,8 @@
       <c r="H204" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I204" s="36">
-        <v>43.6</v>
+      <c r="I204" s="27">
+        <v>10.9</v>
       </c>
       <c r="J204" s="25" t="s">
         <v>377</v>
@@ -14762,11 +14714,11 @@
       </c>
       <c r="N204" s="30">
         <f t="shared" si="8"/>
-        <v>17.440000000000001</v>
+        <v>4.3600000000000003</v>
       </c>
       <c r="O204" s="30">
         <f t="shared" si="9"/>
-        <v>18.137600000000003</v>
+        <v>4.5344000000000007</v>
       </c>
       <c r="P204" s="8"/>
       <c r="Q204" s="50">
@@ -14859,8 +14811,8 @@
       <c r="H206" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I206" s="36">
-        <v>43.6</v>
+      <c r="I206" s="27">
+        <v>10.9</v>
       </c>
       <c r="J206" s="25" t="s">
         <v>377</v>
@@ -14874,11 +14826,11 @@
       </c>
       <c r="N206" s="30">
         <f t="shared" si="8"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O206" s="30">
         <f t="shared" si="9"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P206" s="8"/>
       <c r="Q206" s="50">
@@ -14915,8 +14867,8 @@
       <c r="H207" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I207" s="36">
-        <v>43.6</v>
+      <c r="I207" s="27">
+        <v>10.9</v>
       </c>
       <c r="J207" s="25" t="s">
         <v>377</v>
@@ -14930,11 +14882,11 @@
       </c>
       <c r="N207" s="30">
         <f t="shared" si="8"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O207" s="30">
         <f t="shared" si="9"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P207" s="8"/>
       <c r="Q207" s="50">
@@ -14971,8 +14923,8 @@
       <c r="H208" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I208" s="36">
-        <v>43.6</v>
+      <c r="I208" s="27">
+        <v>10.9</v>
       </c>
       <c r="J208" s="25" t="s">
         <v>377</v>
@@ -14986,11 +14938,11 @@
       </c>
       <c r="N208" s="30">
         <f t="shared" si="8"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O208" s="30">
         <f t="shared" si="9"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P208" s="8"/>
       <c r="Q208" s="50">
@@ -15027,8 +14979,8 @@
       <c r="H209" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I209" s="36">
-        <v>43.6</v>
+      <c r="I209" s="27">
+        <v>10.9</v>
       </c>
       <c r="J209" s="25" t="s">
         <v>377</v>
@@ -15042,11 +14994,11 @@
       </c>
       <c r="N209" s="30">
         <f t="shared" ref="N209:N272" si="12">I209*(1-M209)</f>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O209" s="30">
         <f t="shared" ref="O209:O272" si="13">N209*(1+J209)</f>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P209" s="8"/>
       <c r="Q209" s="50">
@@ -15083,8 +15035,8 @@
       <c r="H210" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I210" s="36">
-        <v>43.6</v>
+      <c r="I210" s="27">
+        <v>10.9</v>
       </c>
       <c r="J210" s="25" t="s">
         <v>377</v>
@@ -15098,11 +15050,11 @@
       </c>
       <c r="N210" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O210" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P210" s="8"/>
       <c r="Q210" s="50">
@@ -15139,8 +15091,8 @@
       <c r="H211" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I211" s="36">
-        <v>43.6</v>
+      <c r="I211" s="27">
+        <v>10.9</v>
       </c>
       <c r="J211" s="25" t="s">
         <v>377</v>
@@ -15154,11 +15106,11 @@
       </c>
       <c r="N211" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O211" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P211" s="8"/>
       <c r="Q211" s="50">
@@ -15251,8 +15203,8 @@
       <c r="H213" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I213" s="36">
-        <v>43.6</v>
+      <c r="I213" s="27">
+        <v>10.9</v>
       </c>
       <c r="J213" s="25" t="s">
         <v>377</v>
@@ -15266,11 +15218,11 @@
       </c>
       <c r="N213" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O213" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P213" s="8"/>
       <c r="Q213" s="50">
@@ -15307,8 +15259,8 @@
       <c r="H214" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I214" s="36">
-        <v>43.6</v>
+      <c r="I214" s="27">
+        <v>10.9</v>
       </c>
       <c r="J214" s="25" t="s">
         <v>377</v>
@@ -15322,11 +15274,11 @@
       </c>
       <c r="N214" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O214" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P214" s="8"/>
       <c r="Q214" s="50">
@@ -15363,8 +15315,8 @@
       <c r="H215" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I215" s="36">
-        <v>43.6</v>
+      <c r="I215" s="27">
+        <v>10.9</v>
       </c>
       <c r="J215" s="25" t="s">
         <v>377</v>
@@ -15378,11 +15330,11 @@
       </c>
       <c r="N215" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O215" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P215" s="8"/>
       <c r="Q215" s="50">
@@ -15419,8 +15371,8 @@
       <c r="H216" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I216" s="36">
-        <v>43.6</v>
+      <c r="I216" s="27">
+        <v>10.9</v>
       </c>
       <c r="J216" s="25" t="s">
         <v>377</v>
@@ -15434,11 +15386,11 @@
       </c>
       <c r="N216" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O216" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P216" s="8"/>
       <c r="Q216" s="50">
@@ -15475,8 +15427,8 @@
       <c r="H217" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I217" s="36">
-        <v>43.6</v>
+      <c r="I217" s="27">
+        <v>10.9</v>
       </c>
       <c r="J217" s="25" t="s">
         <v>377</v>
@@ -15490,11 +15442,11 @@
       </c>
       <c r="N217" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O217" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P217" s="8"/>
       <c r="Q217" s="50">
@@ -15531,8 +15483,8 @@
       <c r="H218" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I218" s="36">
-        <v>43.6</v>
+      <c r="I218" s="27">
+        <v>10.9</v>
       </c>
       <c r="J218" s="25" t="s">
         <v>377</v>
@@ -15546,11 +15498,11 @@
       </c>
       <c r="N218" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O218" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P218" s="8"/>
       <c r="Q218" s="50">
@@ -15643,8 +15595,8 @@
       <c r="H220" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I220" s="36">
-        <v>43.6</v>
+      <c r="I220" s="27">
+        <v>10.9</v>
       </c>
       <c r="J220" s="25" t="s">
         <v>377</v>
@@ -15658,11 +15610,11 @@
       </c>
       <c r="N220" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O220" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P220" s="8"/>
       <c r="Q220" s="50">
@@ -15699,8 +15651,8 @@
       <c r="H221" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I221" s="36">
-        <v>43.6</v>
+      <c r="I221" s="27">
+        <v>10.9</v>
       </c>
       <c r="J221" s="25" t="s">
         <v>377</v>
@@ -15714,11 +15666,11 @@
       </c>
       <c r="N221" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O221" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P221" s="8"/>
       <c r="Q221" s="50">
@@ -15755,8 +15707,8 @@
       <c r="H222" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I222" s="36">
-        <v>43.6</v>
+      <c r="I222" s="27">
+        <v>10.9</v>
       </c>
       <c r="J222" s="25" t="s">
         <v>377</v>
@@ -15770,11 +15722,11 @@
       </c>
       <c r="N222" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O222" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P222" s="8"/>
       <c r="Q222" s="50">
@@ -15811,8 +15763,8 @@
       <c r="H223" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I223" s="36">
-        <v>43.6</v>
+      <c r="I223" s="27">
+        <v>10.9</v>
       </c>
       <c r="J223" s="25" t="s">
         <v>377</v>
@@ -15826,11 +15778,11 @@
       </c>
       <c r="N223" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O223" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P223" s="8"/>
       <c r="Q223" s="50">
@@ -15867,8 +15819,8 @@
       <c r="H224" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I224" s="36">
-        <v>43.6</v>
+      <c r="I224" s="27">
+        <v>10.9</v>
       </c>
       <c r="J224" s="25" t="s">
         <v>377</v>
@@ -15882,11 +15834,11 @@
       </c>
       <c r="N224" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O224" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P224" s="8"/>
       <c r="Q224" s="50">
@@ -15923,8 +15875,8 @@
       <c r="H225" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I225" s="36">
-        <v>43.6</v>
+      <c r="I225" s="27">
+        <v>10.9</v>
       </c>
       <c r="J225" s="25" t="s">
         <v>377</v>
@@ -15938,11 +15890,11 @@
       </c>
       <c r="N225" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O225" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P225" s="8"/>
       <c r="Q225" s="50">
@@ -16035,8 +15987,8 @@
       <c r="H227" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I227" s="36">
-        <v>43.6</v>
+      <c r="I227" s="27">
+        <v>10.9</v>
       </c>
       <c r="J227" s="25" t="s">
         <v>377</v>
@@ -16050,11 +16002,11 @@
       </c>
       <c r="N227" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O227" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P227" s="8"/>
       <c r="Q227" s="50">
@@ -16091,8 +16043,8 @@
       <c r="H228" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I228" s="36">
-        <v>43.6</v>
+      <c r="I228" s="27">
+        <v>10.9</v>
       </c>
       <c r="J228" s="25" t="s">
         <v>377</v>
@@ -16106,11 +16058,11 @@
       </c>
       <c r="N228" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O228" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P228" s="8"/>
       <c r="Q228" s="50">
@@ -16147,8 +16099,8 @@
       <c r="H229" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I229" s="36">
-        <v>43.6</v>
+      <c r="I229" s="27">
+        <v>10.9</v>
       </c>
       <c r="J229" s="25" t="s">
         <v>377</v>
@@ -16162,11 +16114,11 @@
       </c>
       <c r="N229" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O229" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P229" s="8"/>
       <c r="Q229" s="50">
@@ -16203,8 +16155,8 @@
       <c r="H230" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I230" s="36">
-        <v>43.6</v>
+      <c r="I230" s="27">
+        <v>10.9</v>
       </c>
       <c r="J230" s="25" t="s">
         <v>377</v>
@@ -16218,11 +16170,11 @@
       </c>
       <c r="N230" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O230" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P230" s="8"/>
       <c r="Q230" s="50">
@@ -16259,8 +16211,8 @@
       <c r="H231" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I231" s="36">
-        <v>43.6</v>
+      <c r="I231" s="27">
+        <v>10.9</v>
       </c>
       <c r="J231" s="25" t="s">
         <v>377</v>
@@ -16274,11 +16226,11 @@
       </c>
       <c r="N231" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O231" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P231" s="8"/>
       <c r="Q231" s="50">
@@ -16315,8 +16267,8 @@
       <c r="H232" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I232" s="36">
-        <v>43.6</v>
+      <c r="I232" s="27">
+        <v>10.9</v>
       </c>
       <c r="J232" s="25" t="s">
         <v>377</v>
@@ -16330,11 +16282,11 @@
       </c>
       <c r="N232" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O232" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P232" s="8"/>
       <c r="Q232" s="50">
@@ -16427,8 +16379,8 @@
       <c r="H234" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I234" s="36">
-        <v>43.6</v>
+      <c r="I234" s="27">
+        <v>10.9</v>
       </c>
       <c r="J234" s="25" t="s">
         <v>377</v>
@@ -16442,11 +16394,11 @@
       </c>
       <c r="N234" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O234" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P234" s="8"/>
       <c r="Q234" s="50">
@@ -16483,8 +16435,8 @@
       <c r="H235" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I235" s="36">
-        <v>43.6</v>
+      <c r="I235" s="27">
+        <v>10.9</v>
       </c>
       <c r="J235" s="25" t="s">
         <v>377</v>
@@ -16498,11 +16450,11 @@
       </c>
       <c r="N235" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O235" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P235" s="8"/>
       <c r="Q235" s="50">
@@ -16539,8 +16491,8 @@
       <c r="H236" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I236" s="36">
-        <v>43.6</v>
+      <c r="I236" s="27">
+        <v>10.9</v>
       </c>
       <c r="J236" s="25" t="s">
         <v>377</v>
@@ -16554,11 +16506,11 @@
       </c>
       <c r="N236" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O236" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P236" s="8"/>
       <c r="Q236" s="50">
@@ -16595,8 +16547,8 @@
       <c r="H237" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I237" s="36">
-        <v>43.6</v>
+      <c r="I237" s="27">
+        <v>10.9</v>
       </c>
       <c r="J237" s="25" t="s">
         <v>377</v>
@@ -16610,11 +16562,11 @@
       </c>
       <c r="N237" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O237" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P237" s="8"/>
       <c r="Q237" s="50">
@@ -16651,8 +16603,8 @@
       <c r="H238" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I238" s="36">
-        <v>43.6</v>
+      <c r="I238" s="27">
+        <v>10.9</v>
       </c>
       <c r="J238" s="25" t="s">
         <v>377</v>
@@ -16666,11 +16618,11 @@
       </c>
       <c r="N238" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O238" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P238" s="8"/>
       <c r="Q238" s="50">
@@ -16707,8 +16659,8 @@
       <c r="H239" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I239" s="36">
-        <v>43.6</v>
+      <c r="I239" s="27">
+        <v>10.9</v>
       </c>
       <c r="J239" s="25" t="s">
         <v>377</v>
@@ -16722,11 +16674,11 @@
       </c>
       <c r="N239" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O239" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P239" s="8"/>
       <c r="Q239" s="50">
@@ -16819,8 +16771,8 @@
       <c r="H241" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I241" s="36">
-        <v>43.6</v>
+      <c r="I241" s="27">
+        <v>10.9</v>
       </c>
       <c r="J241" s="25" t="s">
         <v>377</v>
@@ -16834,11 +16786,11 @@
       </c>
       <c r="N241" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O241" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P241" s="8"/>
       <c r="Q241" s="50">
@@ -16875,8 +16827,8 @@
       <c r="H242" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I242" s="36">
-        <v>43.6</v>
+      <c r="I242" s="27">
+        <v>10.9</v>
       </c>
       <c r="J242" s="25" t="s">
         <v>377</v>
@@ -16890,11 +16842,11 @@
       </c>
       <c r="N242" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O242" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P242" s="8"/>
       <c r="Q242" s="50">
@@ -16931,8 +16883,8 @@
       <c r="H243" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I243" s="36">
-        <v>43.6</v>
+      <c r="I243" s="27">
+        <v>10.9</v>
       </c>
       <c r="J243" s="25" t="s">
         <v>377</v>
@@ -16946,11 +16898,11 @@
       </c>
       <c r="N243" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O243" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P243" s="8"/>
       <c r="Q243" s="50">
@@ -16987,8 +16939,8 @@
       <c r="H244" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I244" s="36">
-        <v>43.6</v>
+      <c r="I244" s="27">
+        <v>10.9</v>
       </c>
       <c r="J244" s="25" t="s">
         <v>377</v>
@@ -17002,11 +16954,11 @@
       </c>
       <c r="N244" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O244" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P244" s="8"/>
       <c r="Q244" s="50">
@@ -17043,8 +16995,8 @@
       <c r="H245" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I245" s="36">
-        <v>43.6</v>
+      <c r="I245" s="27">
+        <v>10.9</v>
       </c>
       <c r="J245" s="25" t="s">
         <v>377</v>
@@ -17058,11 +17010,11 @@
       </c>
       <c r="N245" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O245" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P245" s="8"/>
       <c r="Q245" s="50">
@@ -17099,8 +17051,8 @@
       <c r="H246" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I246" s="36">
-        <v>43.6</v>
+      <c r="I246" s="27">
+        <v>10.9</v>
       </c>
       <c r="J246" s="25" t="s">
         <v>377</v>
@@ -17114,11 +17066,11 @@
       </c>
       <c r="N246" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O246" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P246" s="8"/>
       <c r="Q246" s="50">
@@ -17211,8 +17163,8 @@
       <c r="H248" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I248" s="36">
-        <v>43.6</v>
+      <c r="I248" s="27">
+        <v>10.9</v>
       </c>
       <c r="J248" s="25" t="s">
         <v>377</v>
@@ -17226,11 +17178,11 @@
       </c>
       <c r="N248" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O248" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P248" s="8"/>
       <c r="Q248" s="50">
@@ -17267,8 +17219,8 @@
       <c r="H249" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I249" s="36">
-        <v>43.6</v>
+      <c r="I249" s="27">
+        <v>10.9</v>
       </c>
       <c r="J249" s="25" t="s">
         <v>377</v>
@@ -17282,11 +17234,11 @@
       </c>
       <c r="N249" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O249" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P249" s="8"/>
       <c r="Q249" s="50">
@@ -17323,8 +17275,8 @@
       <c r="H250" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I250" s="36">
-        <v>43.6</v>
+      <c r="I250" s="27">
+        <v>10.9</v>
       </c>
       <c r="J250" s="25" t="s">
         <v>377</v>
@@ -17338,11 +17290,11 @@
       </c>
       <c r="N250" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O250" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P250" s="8"/>
       <c r="Q250" s="50">
@@ -17379,8 +17331,8 @@
       <c r="H251" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I251" s="36">
-        <v>43.6</v>
+      <c r="I251" s="27">
+        <v>10.9</v>
       </c>
       <c r="J251" s="25" t="s">
         <v>377</v>
@@ -17394,11 +17346,11 @@
       </c>
       <c r="N251" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O251" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P251" s="8"/>
       <c r="Q251" s="50">
@@ -17435,8 +17387,8 @@
       <c r="H252" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I252" s="36">
-        <v>43.6</v>
+      <c r="I252" s="27">
+        <v>10.9</v>
       </c>
       <c r="J252" s="25" t="s">
         <v>377</v>
@@ -17450,11 +17402,11 @@
       </c>
       <c r="N252" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O252" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P252" s="8"/>
       <c r="Q252" s="50">
@@ -17491,8 +17443,8 @@
       <c r="H253" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I253" s="36">
-        <v>43.6</v>
+      <c r="I253" s="27">
+        <v>10.9</v>
       </c>
       <c r="J253" s="25" t="s">
         <v>377</v>
@@ -17506,11 +17458,11 @@
       </c>
       <c r="N253" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O253" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P253" s="8"/>
       <c r="Q253" s="50">
@@ -17603,8 +17555,8 @@
       <c r="H255" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I255" s="36">
-        <v>43.6</v>
+      <c r="I255" s="27">
+        <v>10.9</v>
       </c>
       <c r="J255" s="25" t="s">
         <v>377</v>
@@ -17618,11 +17570,11 @@
       </c>
       <c r="N255" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O255" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P255" s="8"/>
       <c r="Q255" s="50">
@@ -17659,8 +17611,8 @@
       <c r="H256" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I256" s="36">
-        <v>43.6</v>
+      <c r="I256" s="27">
+        <v>10.9</v>
       </c>
       <c r="J256" s="25" t="s">
         <v>377</v>
@@ -17674,11 +17626,11 @@
       </c>
       <c r="N256" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O256" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P256" s="8"/>
       <c r="Q256" s="50">
@@ -17715,8 +17667,8 @@
       <c r="H257" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I257" s="36">
-        <v>43.6</v>
+      <c r="I257" s="27">
+        <v>10.9</v>
       </c>
       <c r="J257" s="25" t="s">
         <v>377</v>
@@ -17730,11 +17682,11 @@
       </c>
       <c r="N257" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O257" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P257" s="8"/>
       <c r="Q257" s="50">
@@ -17771,8 +17723,8 @@
       <c r="H258" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I258" s="36">
-        <v>43.6</v>
+      <c r="I258" s="27">
+        <v>10.9</v>
       </c>
       <c r="J258" s="25" t="s">
         <v>377</v>
@@ -17786,11 +17738,11 @@
       </c>
       <c r="N258" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O258" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P258" s="8"/>
       <c r="Q258" s="50">
@@ -17827,8 +17779,8 @@
       <c r="H259" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I259" s="36">
-        <v>43.6</v>
+      <c r="I259" s="27">
+        <v>10.9</v>
       </c>
       <c r="J259" s="25" t="s">
         <v>377</v>
@@ -17842,11 +17794,11 @@
       </c>
       <c r="N259" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O259" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P259" s="8"/>
       <c r="Q259" s="50">
@@ -17883,8 +17835,8 @@
       <c r="H260" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I260" s="36">
-        <v>43.6</v>
+      <c r="I260" s="27">
+        <v>10.9</v>
       </c>
       <c r="J260" s="25" t="s">
         <v>377</v>
@@ -17898,11 +17850,11 @@
       </c>
       <c r="N260" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O260" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P260" s="8"/>
       <c r="Q260" s="50">
@@ -17995,8 +17947,8 @@
       <c r="H262" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I262" s="36">
-        <v>43.6</v>
+      <c r="I262" s="27">
+        <v>10.9</v>
       </c>
       <c r="J262" s="25" t="s">
         <v>377</v>
@@ -18010,11 +17962,11 @@
       </c>
       <c r="N262" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O262" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P262" s="8"/>
       <c r="Q262" s="50">
@@ -18051,8 +18003,8 @@
       <c r="H263" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I263" s="36">
-        <v>43.6</v>
+      <c r="I263" s="27">
+        <v>10.9</v>
       </c>
       <c r="J263" s="25" t="s">
         <v>377</v>
@@ -18066,11 +18018,11 @@
       </c>
       <c r="N263" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O263" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P263" s="8"/>
       <c r="Q263" s="50">
@@ -18107,8 +18059,8 @@
       <c r="H264" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I264" s="36">
-        <v>43.6</v>
+      <c r="I264" s="27">
+        <v>10.9</v>
       </c>
       <c r="J264" s="25" t="s">
         <v>377</v>
@@ -18122,11 +18074,11 @@
       </c>
       <c r="N264" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O264" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P264" s="8"/>
       <c r="Q264" s="50">
@@ -18163,8 +18115,8 @@
       <c r="H265" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I265" s="36">
-        <v>43.6</v>
+      <c r="I265" s="27">
+        <v>10.9</v>
       </c>
       <c r="J265" s="25" t="s">
         <v>377</v>
@@ -18178,11 +18130,11 @@
       </c>
       <c r="N265" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O265" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P265" s="8"/>
       <c r="Q265" s="50">
@@ -18219,8 +18171,8 @@
       <c r="H266" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I266" s="36">
-        <v>43.6</v>
+      <c r="I266" s="27">
+        <v>10.9</v>
       </c>
       <c r="J266" s="25" t="s">
         <v>377</v>
@@ -18234,11 +18186,11 @@
       </c>
       <c r="N266" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O266" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P266" s="8"/>
       <c r="Q266" s="50">
@@ -18275,8 +18227,8 @@
       <c r="H267" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I267" s="36">
-        <v>43.6</v>
+      <c r="I267" s="27">
+        <v>10.9</v>
       </c>
       <c r="J267" s="25" t="s">
         <v>377</v>
@@ -18290,11 +18242,11 @@
       </c>
       <c r="N267" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O267" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P267" s="8"/>
       <c r="Q267" s="50">
@@ -18387,8 +18339,8 @@
       <c r="H269" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I269" s="36">
-        <v>43.6</v>
+      <c r="I269" s="27">
+        <v>10.9</v>
       </c>
       <c r="J269" s="25" t="s">
         <v>377</v>
@@ -18402,11 +18354,11 @@
       </c>
       <c r="N269" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O269" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P269" s="8"/>
       <c r="Q269" s="50">
@@ -18443,8 +18395,8 @@
       <c r="H270" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I270" s="36">
-        <v>43.6</v>
+      <c r="I270" s="27">
+        <v>10.9</v>
       </c>
       <c r="J270" s="25" t="s">
         <v>377</v>
@@ -18458,11 +18410,11 @@
       </c>
       <c r="N270" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O270" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P270" s="8"/>
       <c r="Q270" s="50">
@@ -18499,8 +18451,8 @@
       <c r="H271" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I271" s="36">
-        <v>43.6</v>
+      <c r="I271" s="27">
+        <v>10.9</v>
       </c>
       <c r="J271" s="25" t="s">
         <v>377</v>
@@ -18514,11 +18466,11 @@
       </c>
       <c r="N271" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O271" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P271" s="8"/>
       <c r="Q271" s="50">
@@ -18555,8 +18507,8 @@
       <c r="H272" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I272" s="36">
-        <v>43.6</v>
+      <c r="I272" s="27">
+        <v>10.9</v>
       </c>
       <c r="J272" s="25" t="s">
         <v>377</v>
@@ -18570,11 +18522,11 @@
       </c>
       <c r="N272" s="30">
         <f t="shared" si="12"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O272" s="30">
         <f t="shared" si="13"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P272" s="8"/>
       <c r="Q272" s="50">
@@ -18611,8 +18563,8 @@
       <c r="H273" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I273" s="36">
-        <v>43.6</v>
+      <c r="I273" s="27">
+        <v>10.9</v>
       </c>
       <c r="J273" s="25" t="s">
         <v>377</v>
@@ -18626,11 +18578,11 @@
       </c>
       <c r="N273" s="30">
         <f t="shared" ref="N273:N281" si="16">I273*(1-M273)</f>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O273" s="30">
         <f t="shared" ref="O273:O290" si="17">N273*(1+J273)</f>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P273" s="8"/>
       <c r="Q273" s="50">
@@ -18667,8 +18619,8 @@
       <c r="H274" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I274" s="36">
-        <v>43.6</v>
+      <c r="I274" s="27">
+        <v>10.9</v>
       </c>
       <c r="J274" s="25" t="s">
         <v>377</v>
@@ -18682,11 +18634,11 @@
       </c>
       <c r="N274" s="30">
         <f t="shared" si="16"/>
-        <v>21.8</v>
+        <v>5.45</v>
       </c>
       <c r="O274" s="30">
         <f t="shared" si="17"/>
-        <v>22.672000000000001</v>
+        <v>5.6680000000000001</v>
       </c>
       <c r="P274" s="8"/>
       <c r="Q274" s="50">
@@ -18871,33 +18823,33 @@
         <v>177</v>
       </c>
       <c r="B278" s="16" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="C278" s="16" t="s">
+        <v>698</v>
+      </c>
+      <c r="D278" s="31" t="s">
+        <v>696</v>
+      </c>
+      <c r="E278" s="31" t="s">
+        <v>697</v>
+      </c>
+      <c r="F278" s="32" t="s">
         <v>699</v>
       </c>
-      <c r="D278" s="31" t="s">
-        <v>697</v>
-      </c>
-      <c r="E278" s="94" t="s">
-        <v>698</v>
-      </c>
-      <c r="F278" s="95" t="s">
-        <v>700</v>
-      </c>
-      <c r="G278" s="95" t="s">
+      <c r="G278" s="32" t="s">
         <v>193</v>
       </c>
-      <c r="H278" s="95" t="s">
-        <v>191</v>
-      </c>
-      <c r="I278" s="96">
+      <c r="H278" s="32" t="s">
+        <v>191</v>
+      </c>
+      <c r="I278" s="33">
         <v>103.2</v>
       </c>
-      <c r="J278" s="95" t="s">
+      <c r="J278" s="32" t="s">
         <v>378</v>
       </c>
-      <c r="K278" s="38">
+      <c r="K278" s="34">
         <v>8052747326532</v>
       </c>
       <c r="L278" s="38" t="s">
@@ -18906,11 +18858,11 @@
       <c r="M278" s="29">
         <v>0.6</v>
       </c>
-      <c r="N278" s="92">
+      <c r="N278" s="23">
         <f t="shared" si="16"/>
         <v>41.28</v>
       </c>
-      <c r="O278" s="92">
+      <c r="O278" s="23">
         <f t="shared" si="17"/>
         <v>50.361600000000003</v>
       </c>
@@ -19270,35 +19222,35 @@
       <c r="D285" s="35">
         <v>1812</v>
       </c>
-      <c r="E285" s="87" t="s">
-        <v>696</v>
-      </c>
-      <c r="F285" s="87" t="s">
+      <c r="E285" s="35" t="s">
+        <v>695</v>
+      </c>
+      <c r="F285" s="35" t="s">
         <v>365</v>
       </c>
-      <c r="G285" s="89" t="s">
-        <v>191</v>
-      </c>
-      <c r="H285" s="89" t="s">
-        <v>191</v>
-      </c>
-      <c r="I285" s="90">
+      <c r="G285" s="25" t="s">
+        <v>191</v>
+      </c>
+      <c r="H285" s="25" t="s">
+        <v>191</v>
+      </c>
+      <c r="I285" s="36">
         <v>75</v>
       </c>
-      <c r="J285" s="89" t="s">
+      <c r="J285" s="25" t="s">
         <v>378</v>
       </c>
-      <c r="K285" s="91">
+      <c r="K285" s="37">
         <v>8058032048615</v>
       </c>
-      <c r="L285" s="91"/>
-      <c r="M285" s="91" t="s">
+      <c r="L285" s="37"/>
+      <c r="M285" s="37" t="s">
         <v>683</v>
       </c>
-      <c r="N285" s="90">
+      <c r="N285" s="36">
         <v>75</v>
       </c>
-      <c r="O285" s="92">
+      <c r="O285" s="30">
         <f t="shared" si="17"/>
         <v>91.5</v>
       </c>
@@ -19381,7 +19333,7 @@
         <v>1781</v>
       </c>
       <c r="E287" s="16" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="F287" s="16" t="s">
         <v>365</v>
@@ -19399,7 +19351,7 @@
         <v>378</v>
       </c>
       <c r="K287" s="16" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="L287" s="16"/>
       <c r="M287" s="16" t="s">
@@ -19436,7 +19388,7 @@
         <v>1783</v>
       </c>
       <c r="E288" s="16" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="F288" s="16" t="s">
         <v>365</v>
@@ -19454,7 +19406,7 @@
         <v>378</v>
       </c>
       <c r="K288" s="16" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="L288" s="16"/>
       <c r="M288" s="16" t="s">
@@ -19490,35 +19442,35 @@
       <c r="D289" s="16">
         <v>1813</v>
       </c>
-      <c r="E289" s="88" t="s">
-        <v>707</v>
-      </c>
-      <c r="F289" s="88" t="s">
+      <c r="E289" s="16" t="s">
+        <v>706</v>
+      </c>
+      <c r="F289" s="16" t="s">
         <v>365</v>
       </c>
-      <c r="G289" s="88">
+      <c r="G289" s="16">
         <v>1</v>
       </c>
-      <c r="H289" s="88">
+      <c r="H289" s="16">
         <v>1</v>
       </c>
-      <c r="I289" s="90">
+      <c r="I289" s="36">
         <v>75</v>
       </c>
-      <c r="J289" s="88" t="s">
+      <c r="J289" s="16" t="s">
         <v>378</v>
       </c>
-      <c r="K289" s="93">
+      <c r="K289" s="52">
         <v>8058032048622</v>
       </c>
-      <c r="L289" s="88"/>
-      <c r="M289" s="88" t="s">
+      <c r="L289" s="16"/>
+      <c r="M289" s="16" t="s">
         <v>683</v>
       </c>
-      <c r="N289" s="90">
+      <c r="N289" s="36">
         <v>75</v>
       </c>
-      <c r="O289" s="92">
+      <c r="O289" s="30">
         <f t="shared" si="17"/>
         <v>91.5</v>
       </c>
@@ -19546,7 +19498,7 @@
         <v>1590</v>
       </c>
       <c r="E290" s="16" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="F290" s="16" t="s">
         <v>365</v>
@@ -19564,7 +19516,7 @@
         <v>378</v>
       </c>
       <c r="K290" s="16" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="L290" s="16"/>
       <c r="M290" s="16" t="s">
@@ -19645,14 +19597,14 @@
       <c r="K293" s="43"/>
       <c r="L293" s="43"/>
       <c r="M293" s="43"/>
-      <c r="N293" s="55" t="s">
-        <v>690</v>
-      </c>
-      <c r="O293" s="56"/>
-      <c r="Q293" s="60" t="s">
-        <v>694</v>
-      </c>
-      <c r="R293" s="63">
+      <c r="N293" s="83" t="s">
+        <v>689</v>
+      </c>
+      <c r="O293" s="84"/>
+      <c r="Q293" s="65" t="s">
+        <v>693</v>
+      </c>
+      <c r="R293" s="68">
         <f>R291+N297</f>
         <v>11.59</v>
       </c>
@@ -19678,8 +19630,8 @@
         <f>MIN(MAX(Q291*N294,9.5),99)</f>
         <v>9.5</v>
       </c>
-      <c r="Q294" s="61"/>
-      <c r="R294" s="64"/>
+      <c r="Q294" s="66"/>
+      <c r="R294" s="69"/>
     </row>
     <row r="295" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A295" s="43"/>
@@ -19695,12 +19647,12 @@
       <c r="K295" s="43"/>
       <c r="L295" s="43"/>
       <c r="M295" s="43"/>
-      <c r="N295" s="57" t="s">
-        <v>693</v>
-      </c>
-      <c r="O295" s="58"/>
-      <c r="Q295" s="61"/>
-      <c r="R295" s="64"/>
+      <c r="N295" s="85" t="s">
+        <v>692</v>
+      </c>
+      <c r="O295" s="86"/>
+      <c r="Q295" s="66"/>
+      <c r="R295" s="69"/>
     </row>
     <row r="296" spans="1:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A296" s="43"/>
@@ -19723,8 +19675,8 @@
         <f>O294*N296</f>
         <v>2.09</v>
       </c>
-      <c r="Q296" s="62"/>
-      <c r="R296" s="65"/>
+      <c r="Q296" s="67"/>
+      <c r="R296" s="70"/>
     </row>
     <row r="297" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A297" s="43"/>
@@ -19740,14 +19692,29 @@
       <c r="K297" s="43"/>
       <c r="L297" s="43"/>
       <c r="M297" s="43"/>
-      <c r="N297" s="59">
+      <c r="N297" s="87">
         <f>O294+O296</f>
         <v>11.59</v>
       </c>
-      <c r="O297" s="59"/>
+      <c r="O297" s="87"/>
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="I7:P7"/>
+    <mergeCell ref="I6:P6"/>
+    <mergeCell ref="N293:O293"/>
+    <mergeCell ref="N295:O295"/>
+    <mergeCell ref="N297:O297"/>
+    <mergeCell ref="Q293:Q296"/>
+    <mergeCell ref="R293:R296"/>
+    <mergeCell ref="D12:G12"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="H8:H12"/>
+    <mergeCell ref="I8:P12"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="D10:G10"/>
     <mergeCell ref="A2:P2"/>
     <mergeCell ref="A13:P13"/>
     <mergeCell ref="A7:C7"/>
@@ -19764,21 +19731,6 @@
     <mergeCell ref="D11:G11"/>
     <mergeCell ref="D7:G7"/>
     <mergeCell ref="A12:C12"/>
-    <mergeCell ref="Q293:Q296"/>
-    <mergeCell ref="R293:R296"/>
-    <mergeCell ref="D12:G12"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="D8:G8"/>
-    <mergeCell ref="H8:H12"/>
-    <mergeCell ref="I8:P12"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="D10:G10"/>
-    <mergeCell ref="I7:P7"/>
-    <mergeCell ref="I6:P6"/>
-    <mergeCell ref="N293:O293"/>
-    <mergeCell ref="N295:O295"/>
-    <mergeCell ref="N297:O297"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Revert "Nuovo ordine_template.xlsx + niente cache CDN sul template di lavoro"
This reverts commit 37f4e426bfea8c31767cfec9e741272d355bee02.
</commit_message>
<xml_diff>
--- a/ordine_template.xlsx
+++ b/ordine_template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GRAFICA\GRAFICA 2026\programma occhiali detomaso\09 09 2026 inserimento 3 NUOVI ARTICOLI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC_Graphic\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7DE9FA84-36F5-4EB6-A9ED-AAD402438EDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A54806A9-E677-4C33-A913-2BC90280081B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{1DF05D46-8AE3-4E7B-8533-2DA2E4746004}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2577" uniqueCount="707">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2586" uniqueCount="708">
   <si>
     <t>CODICE</t>
   </si>
@@ -2100,6 +2100,9 @@
   </si>
   <si>
     <t>PROVINCIA:</t>
+  </si>
+  <si>
+    <t>OBBLIGATORIO</t>
   </si>
   <si>
     <t>CELLULARE:</t>
@@ -2628,7 +2631,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
@@ -2794,43 +2797,6 @@
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -2842,6 +2808,21 @@
     <xf numFmtId="0" fontId="9" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="5" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="5" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="6" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="12" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2860,6 +2841,30 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="12" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2909,19 +2914,44 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="5" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="5" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="6" fillId="6" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3264,256 +3294,274 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:20" s="1" customFormat="1" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="53" t="s">
+      <c r="A2" s="84" t="s">
         <v>367</v>
       </c>
-      <c r="B2" s="54"/>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
-      <c r="I2" s="54"/>
-      <c r="J2" s="54"/>
-      <c r="K2" s="54"/>
-      <c r="L2" s="54"/>
-      <c r="M2" s="54"/>
-      <c r="N2" s="54"/>
-      <c r="O2" s="54"/>
-      <c r="P2" s="54"/>
+      <c r="B2" s="85"/>
+      <c r="C2" s="85"/>
+      <c r="D2" s="85"/>
+      <c r="E2" s="85"/>
+      <c r="F2" s="85"/>
+      <c r="G2" s="85"/>
+      <c r="H2" s="85"/>
+      <c r="I2" s="85"/>
+      <c r="J2" s="85"/>
+      <c r="K2" s="85"/>
+      <c r="L2" s="85"/>
+      <c r="M2" s="85"/>
+      <c r="N2" s="85"/>
+      <c r="O2" s="85"/>
+      <c r="P2" s="85"/>
       <c r="R2" s="2"/>
     </row>
     <row r="3" spans="1:20" s="1" customFormat="1" ht="6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="R3" s="2"/>
     </row>
     <row r="4" spans="1:20" s="1" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="60" t="s">
+      <c r="A4" s="67" t="s">
         <v>686</v>
       </c>
-      <c r="B4" s="61"/>
-      <c r="C4" s="61"/>
-      <c r="D4" s="59"/>
-      <c r="E4" s="59"/>
-      <c r="F4" s="59"/>
-      <c r="G4" s="59"/>
+      <c r="B4" s="68"/>
+      <c r="C4" s="68"/>
+      <c r="D4" s="66" t="s">
+        <v>688</v>
+      </c>
+      <c r="E4" s="66"/>
+      <c r="F4" s="66"/>
+      <c r="G4" s="66"/>
       <c r="H4" s="3" t="s">
         <v>368</v>
       </c>
-      <c r="I4" s="62"/>
-      <c r="J4" s="63"/>
-      <c r="K4" s="63"/>
-      <c r="L4" s="63"/>
-      <c r="M4" s="63"/>
-      <c r="N4" s="63"/>
-      <c r="O4" s="63"/>
-      <c r="P4" s="64"/>
+      <c r="I4" s="52"/>
+      <c r="J4" s="53"/>
+      <c r="K4" s="53"/>
+      <c r="L4" s="53"/>
+      <c r="M4" s="53"/>
+      <c r="N4" s="53"/>
+      <c r="O4" s="53"/>
+      <c r="P4" s="54"/>
       <c r="Q4" s="4"/>
       <c r="R4" s="2"/>
     </row>
     <row r="5" spans="1:20" s="1" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="60" t="s">
+      <c r="A5" s="67" t="s">
         <v>369</v>
       </c>
-      <c r="B5" s="61"/>
-      <c r="C5" s="61"/>
-      <c r="D5" s="59"/>
-      <c r="E5" s="59"/>
-      <c r="F5" s="59"/>
-      <c r="G5" s="59"/>
+      <c r="B5" s="68"/>
+      <c r="C5" s="68"/>
+      <c r="D5" s="66" t="s">
+        <v>688</v>
+      </c>
+      <c r="E5" s="66"/>
+      <c r="F5" s="66"/>
+      <c r="G5" s="66"/>
       <c r="H5" s="3" t="s">
         <v>370</v>
       </c>
-      <c r="I5" s="62"/>
-      <c r="J5" s="63"/>
-      <c r="K5" s="63"/>
-      <c r="L5" s="63"/>
-      <c r="M5" s="63"/>
-      <c r="N5" s="63"/>
-      <c r="O5" s="63"/>
-      <c r="P5" s="64"/>
+      <c r="I5" s="52"/>
+      <c r="J5" s="53"/>
+      <c r="K5" s="53"/>
+      <c r="L5" s="53"/>
+      <c r="M5" s="53"/>
+      <c r="N5" s="53"/>
+      <c r="O5" s="53"/>
+      <c r="P5" s="54"/>
       <c r="Q5" s="4"/>
       <c r="R5" s="2"/>
     </row>
     <row r="6" spans="1:20" s="1" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="56" t="s">
+      <c r="A6" s="69" t="s">
         <v>679</v>
       </c>
-      <c r="B6" s="57"/>
-      <c r="C6" s="58"/>
-      <c r="D6" s="59"/>
-      <c r="E6" s="59"/>
-      <c r="F6" s="59"/>
-      <c r="G6" s="59"/>
+      <c r="B6" s="70"/>
+      <c r="C6" s="71"/>
+      <c r="D6" s="66" t="s">
+        <v>688</v>
+      </c>
+      <c r="E6" s="66"/>
+      <c r="F6" s="66"/>
+      <c r="G6" s="66"/>
       <c r="H6" s="3" t="s">
         <v>372</v>
       </c>
-      <c r="I6" s="62"/>
-      <c r="J6" s="63"/>
-      <c r="K6" s="63"/>
-      <c r="L6" s="63"/>
-      <c r="M6" s="63"/>
-      <c r="N6" s="63"/>
-      <c r="O6" s="63"/>
-      <c r="P6" s="64"/>
+      <c r="I6" s="52"/>
+      <c r="J6" s="53"/>
+      <c r="K6" s="53"/>
+      <c r="L6" s="53"/>
+      <c r="M6" s="53"/>
+      <c r="N6" s="53"/>
+      <c r="O6" s="53"/>
+      <c r="P6" s="54"/>
       <c r="Q6" s="4"/>
       <c r="R6" s="2"/>
     </row>
     <row r="7" spans="1:20" s="1" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="56" t="s">
+      <c r="A7" s="69" t="s">
         <v>680</v>
       </c>
-      <c r="B7" s="57"/>
-      <c r="C7" s="58"/>
-      <c r="D7" s="59"/>
-      <c r="E7" s="59"/>
-      <c r="F7" s="59"/>
-      <c r="G7" s="59"/>
+      <c r="B7" s="70"/>
+      <c r="C7" s="71"/>
+      <c r="D7" s="66" t="s">
+        <v>688</v>
+      </c>
+      <c r="E7" s="66"/>
+      <c r="F7" s="66"/>
+      <c r="G7" s="66"/>
       <c r="H7" s="3" t="s">
         <v>373</v>
       </c>
-      <c r="I7" s="62"/>
-      <c r="J7" s="63"/>
-      <c r="K7" s="63"/>
-      <c r="L7" s="63"/>
-      <c r="M7" s="63"/>
-      <c r="N7" s="63"/>
-      <c r="O7" s="63"/>
-      <c r="P7" s="64"/>
+      <c r="I7" s="52"/>
+      <c r="J7" s="53"/>
+      <c r="K7" s="53"/>
+      <c r="L7" s="53"/>
+      <c r="M7" s="53"/>
+      <c r="N7" s="53"/>
+      <c r="O7" s="53"/>
+      <c r="P7" s="54"/>
       <c r="Q7" s="4"/>
       <c r="R7" s="2"/>
     </row>
     <row r="8" spans="1:20" s="1" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="56" t="s">
+      <c r="A8" s="69" t="s">
         <v>687</v>
       </c>
-      <c r="B8" s="57"/>
-      <c r="C8" s="58"/>
-      <c r="D8" s="59"/>
-      <c r="E8" s="59"/>
-      <c r="F8" s="59"/>
-      <c r="G8" s="59"/>
-      <c r="H8" s="71" t="s">
+      <c r="B8" s="70"/>
+      <c r="C8" s="71"/>
+      <c r="D8" s="66" t="s">
+        <v>688</v>
+      </c>
+      <c r="E8" s="66"/>
+      <c r="F8" s="66"/>
+      <c r="G8" s="66"/>
+      <c r="H8" s="72" t="s">
         <v>375</v>
       </c>
-      <c r="I8" s="74"/>
-      <c r="J8" s="75"/>
-      <c r="K8" s="75"/>
-      <c r="L8" s="75"/>
-      <c r="M8" s="75"/>
-      <c r="N8" s="75"/>
-      <c r="O8" s="75"/>
-      <c r="P8" s="76"/>
+      <c r="I8" s="75"/>
+      <c r="J8" s="76"/>
+      <c r="K8" s="76"/>
+      <c r="L8" s="76"/>
+      <c r="M8" s="76"/>
+      <c r="N8" s="76"/>
+      <c r="O8" s="76"/>
+      <c r="P8" s="77"/>
       <c r="Q8" s="4"/>
       <c r="R8" s="2"/>
     </row>
     <row r="9" spans="1:20" s="1" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="60" t="s">
+      <c r="A9" s="67" t="s">
         <v>371</v>
       </c>
-      <c r="B9" s="61"/>
-      <c r="C9" s="61"/>
-      <c r="D9" s="59"/>
-      <c r="E9" s="59"/>
-      <c r="F9" s="59"/>
-      <c r="G9" s="59"/>
-      <c r="H9" s="72"/>
-      <c r="I9" s="77"/>
-      <c r="J9" s="78"/>
-      <c r="K9" s="78"/>
-      <c r="L9" s="78"/>
-      <c r="M9" s="78"/>
-      <c r="N9" s="78"/>
-      <c r="O9" s="78"/>
-      <c r="P9" s="79"/>
+      <c r="B9" s="68"/>
+      <c r="C9" s="68"/>
+      <c r="D9" s="66" t="s">
+        <v>688</v>
+      </c>
+      <c r="E9" s="66"/>
+      <c r="F9" s="66"/>
+      <c r="G9" s="66"/>
+      <c r="H9" s="73"/>
+      <c r="I9" s="78"/>
+      <c r="J9" s="79"/>
+      <c r="K9" s="79"/>
+      <c r="L9" s="79"/>
+      <c r="M9" s="79"/>
+      <c r="N9" s="79"/>
+      <c r="O9" s="79"/>
+      <c r="P9" s="80"/>
       <c r="Q9" s="4"/>
       <c r="R9" s="2"/>
     </row>
     <row r="10" spans="1:20" s="1" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="56" t="s">
-        <v>694</v>
-      </c>
-      <c r="B10" s="57"/>
-      <c r="C10" s="58"/>
-      <c r="D10" s="59"/>
-      <c r="E10" s="59"/>
-      <c r="F10" s="59"/>
-      <c r="G10" s="59"/>
-      <c r="H10" s="72"/>
-      <c r="I10" s="77"/>
-      <c r="J10" s="78"/>
-      <c r="K10" s="78"/>
-      <c r="L10" s="78"/>
-      <c r="M10" s="78"/>
-      <c r="N10" s="78"/>
-      <c r="O10" s="78"/>
-      <c r="P10" s="79"/>
+      <c r="A10" s="69" t="s">
+        <v>695</v>
+      </c>
+      <c r="B10" s="70"/>
+      <c r="C10" s="71"/>
+      <c r="D10" s="66" t="s">
+        <v>688</v>
+      </c>
+      <c r="E10" s="66"/>
+      <c r="F10" s="66"/>
+      <c r="G10" s="66"/>
+      <c r="H10" s="73"/>
+      <c r="I10" s="78"/>
+      <c r="J10" s="79"/>
+      <c r="K10" s="79"/>
+      <c r="L10" s="79"/>
+      <c r="M10" s="79"/>
+      <c r="N10" s="79"/>
+      <c r="O10" s="79"/>
+      <c r="P10" s="80"/>
       <c r="Q10" s="4"/>
       <c r="R10" s="2"/>
     </row>
     <row r="11" spans="1:20" s="1" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="60" t="s">
+      <c r="A11" s="67" t="s">
+        <v>689</v>
+      </c>
+      <c r="B11" s="68"/>
+      <c r="C11" s="68"/>
+      <c r="D11" s="66" t="s">
         <v>688</v>
       </c>
-      <c r="B11" s="61"/>
-      <c r="C11" s="61"/>
-      <c r="D11" s="59"/>
-      <c r="E11" s="59"/>
-      <c r="F11" s="59"/>
-      <c r="G11" s="59"/>
-      <c r="H11" s="72"/>
-      <c r="I11" s="77"/>
-      <c r="J11" s="78"/>
-      <c r="K11" s="78"/>
-      <c r="L11" s="78"/>
-      <c r="M11" s="78"/>
-      <c r="N11" s="78"/>
-      <c r="O11" s="78"/>
-      <c r="P11" s="79"/>
+      <c r="E11" s="66"/>
+      <c r="F11" s="66"/>
+      <c r="G11" s="66"/>
+      <c r="H11" s="73"/>
+      <c r="I11" s="78"/>
+      <c r="J11" s="79"/>
+      <c r="K11" s="79"/>
+      <c r="L11" s="79"/>
+      <c r="M11" s="79"/>
+      <c r="N11" s="79"/>
+      <c r="O11" s="79"/>
+      <c r="P11" s="80"/>
       <c r="Q11" s="4"/>
       <c r="R11" s="2"/>
     </row>
     <row r="12" spans="1:20" s="1" customFormat="1" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="56" t="s">
+      <c r="A12" s="69" t="s">
         <v>681</v>
       </c>
-      <c r="B12" s="57"/>
-      <c r="C12" s="58"/>
-      <c r="D12" s="59"/>
-      <c r="E12" s="59"/>
-      <c r="F12" s="59"/>
-      <c r="G12" s="59"/>
-      <c r="H12" s="73"/>
-      <c r="I12" s="80"/>
-      <c r="J12" s="81"/>
-      <c r="K12" s="81"/>
-      <c r="L12" s="81"/>
-      <c r="M12" s="81"/>
-      <c r="N12" s="81"/>
-      <c r="O12" s="81"/>
-      <c r="P12" s="82"/>
+      <c r="B12" s="70"/>
+      <c r="C12" s="71"/>
+      <c r="D12" s="66" t="s">
+        <v>688</v>
+      </c>
+      <c r="E12" s="66"/>
+      <c r="F12" s="66"/>
+      <c r="G12" s="66"/>
+      <c r="H12" s="74"/>
+      <c r="I12" s="81"/>
+      <c r="J12" s="82"/>
+      <c r="K12" s="82"/>
+      <c r="L12" s="82"/>
+      <c r="M12" s="82"/>
+      <c r="N12" s="82"/>
+      <c r="O12" s="82"/>
+      <c r="P12" s="83"/>
       <c r="Q12" s="4"/>
       <c r="R12" s="2"/>
     </row>
     <row r="13" spans="1:20" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="55" t="s">
+      <c r="A13" s="86" t="s">
         <v>374</v>
       </c>
-      <c r="B13" s="54"/>
-      <c r="C13" s="54"/>
-      <c r="D13" s="54"/>
-      <c r="E13" s="54"/>
-      <c r="F13" s="54"/>
-      <c r="G13" s="54"/>
-      <c r="H13" s="54"/>
-      <c r="I13" s="54"/>
-      <c r="J13" s="54"/>
-      <c r="K13" s="54"/>
-      <c r="L13" s="54"/>
-      <c r="M13" s="54"/>
-      <c r="N13" s="54"/>
-      <c r="O13" s="54"/>
-      <c r="P13" s="54"/>
+      <c r="B13" s="85"/>
+      <c r="C13" s="85"/>
+      <c r="D13" s="85"/>
+      <c r="E13" s="85"/>
+      <c r="F13" s="85"/>
+      <c r="G13" s="85"/>
+      <c r="H13" s="85"/>
+      <c r="I13" s="85"/>
+      <c r="J13" s="85"/>
+      <c r="K13" s="85"/>
+      <c r="L13" s="85"/>
+      <c r="M13" s="85"/>
+      <c r="N13" s="85"/>
+      <c r="O13" s="85"/>
+      <c r="P13" s="85"/>
       <c r="R13" s="2"/>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.25">
@@ -3566,10 +3614,10 @@
         <v>366</v>
       </c>
       <c r="Q15" s="49" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="R15" s="49" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="S15" s="6"/>
       <c r="T15" s="6"/>
@@ -9477,8 +9525,8 @@
       <c r="H114" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I114" s="27">
-        <v>10.9</v>
+      <c r="I114" s="36">
+        <v>43.6</v>
       </c>
       <c r="J114" s="25" t="s">
         <v>377</v>
@@ -9494,11 +9542,11 @@
       </c>
       <c r="N114" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O114" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P114" s="8"/>
       <c r="Q114" s="50">
@@ -9535,8 +9583,8 @@
       <c r="H115" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I115" s="27">
-        <v>10.9</v>
+      <c r="I115" s="36">
+        <v>43.6</v>
       </c>
       <c r="J115" s="25" t="s">
         <v>377</v>
@@ -9552,11 +9600,11 @@
       </c>
       <c r="N115" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O115" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P115" s="8"/>
       <c r="Q115" s="50">
@@ -9593,8 +9641,8 @@
       <c r="H116" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I116" s="27">
-        <v>10.9</v>
+      <c r="I116" s="36">
+        <v>43.6</v>
       </c>
       <c r="J116" s="25" t="s">
         <v>377</v>
@@ -9610,11 +9658,11 @@
       </c>
       <c r="N116" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O116" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P116" s="8"/>
       <c r="Q116" s="50">
@@ -9651,8 +9699,8 @@
       <c r="H117" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I117" s="27">
-        <v>10.9</v>
+      <c r="I117" s="36">
+        <v>43.6</v>
       </c>
       <c r="J117" s="25" t="s">
         <v>377</v>
@@ -9668,11 +9716,11 @@
       </c>
       <c r="N117" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O117" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P117" s="8"/>
       <c r="Q117" s="50">
@@ -9709,8 +9757,8 @@
       <c r="H118" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I118" s="27">
-        <v>10.9</v>
+      <c r="I118" s="36">
+        <v>43.6</v>
       </c>
       <c r="J118" s="25" t="s">
         <v>377</v>
@@ -9726,11 +9774,11 @@
       </c>
       <c r="N118" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O118" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P118" s="8"/>
       <c r="Q118" s="50">
@@ -9767,8 +9815,8 @@
       <c r="H119" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I119" s="27">
-        <v>10.9</v>
+      <c r="I119" s="36">
+        <v>43.6</v>
       </c>
       <c r="J119" s="25" t="s">
         <v>377</v>
@@ -9784,11 +9832,11 @@
       </c>
       <c r="N119" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O119" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P119" s="8"/>
       <c r="Q119" s="50">
@@ -9825,8 +9873,8 @@
       <c r="H120" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I120" s="27">
-        <v>10.9</v>
+      <c r="I120" s="36">
+        <v>43.6</v>
       </c>
       <c r="J120" s="25" t="s">
         <v>377</v>
@@ -9842,11 +9890,11 @@
       </c>
       <c r="N120" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O120" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P120" s="8"/>
       <c r="Q120" s="50">
@@ -9883,8 +9931,8 @@
       <c r="H121" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I121" s="27">
-        <v>10.9</v>
+      <c r="I121" s="36">
+        <v>43.6</v>
       </c>
       <c r="J121" s="25" t="s">
         <v>377</v>
@@ -9900,11 +9948,11 @@
       </c>
       <c r="N121" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O121" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P121" s="8"/>
       <c r="Q121" s="50">
@@ -9941,8 +9989,8 @@
       <c r="H122" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I122" s="27">
-        <v>10.9</v>
+      <c r="I122" s="36">
+        <v>43.6</v>
       </c>
       <c r="J122" s="25" t="s">
         <v>377</v>
@@ -9958,11 +10006,11 @@
       </c>
       <c r="N122" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O122" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P122" s="8"/>
       <c r="Q122" s="50">
@@ -9999,8 +10047,8 @@
       <c r="H123" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I123" s="27">
-        <v>10.9</v>
+      <c r="I123" s="36">
+        <v>43.6</v>
       </c>
       <c r="J123" s="25" t="s">
         <v>377</v>
@@ -10016,11 +10064,11 @@
       </c>
       <c r="N123" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O123" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P123" s="8"/>
       <c r="Q123" s="50">
@@ -10057,8 +10105,8 @@
       <c r="H124" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I124" s="27">
-        <v>10.9</v>
+      <c r="I124" s="36">
+        <v>43.6</v>
       </c>
       <c r="J124" s="25" t="s">
         <v>377</v>
@@ -10074,11 +10122,11 @@
       </c>
       <c r="N124" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O124" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P124" s="8"/>
       <c r="Q124" s="50">
@@ -10115,8 +10163,8 @@
       <c r="H125" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I125" s="27">
-        <v>10.9</v>
+      <c r="I125" s="36">
+        <v>43.6</v>
       </c>
       <c r="J125" s="25" t="s">
         <v>377</v>
@@ -10132,11 +10180,11 @@
       </c>
       <c r="N125" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O125" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P125" s="8"/>
       <c r="Q125" s="50">
@@ -10173,8 +10221,8 @@
       <c r="H126" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I126" s="27">
-        <v>10.9</v>
+      <c r="I126" s="36">
+        <v>43.6</v>
       </c>
       <c r="J126" s="25" t="s">
         <v>377</v>
@@ -10190,11 +10238,11 @@
       </c>
       <c r="N126" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O126" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P126" s="8"/>
       <c r="Q126" s="50">
@@ -10231,8 +10279,8 @@
       <c r="H127" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I127" s="27">
-        <v>10.9</v>
+      <c r="I127" s="36">
+        <v>43.6</v>
       </c>
       <c r="J127" s="25" t="s">
         <v>377</v>
@@ -10248,11 +10296,11 @@
       </c>
       <c r="N127" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O127" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P127" s="8"/>
       <c r="Q127" s="50">
@@ -10289,8 +10337,8 @@
       <c r="H128" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I128" s="27">
-        <v>10.9</v>
+      <c r="I128" s="36">
+        <v>43.6</v>
       </c>
       <c r="J128" s="25" t="s">
         <v>377</v>
@@ -10306,11 +10354,11 @@
       </c>
       <c r="N128" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O128" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P128" s="8"/>
       <c r="Q128" s="50">
@@ -10347,8 +10395,8 @@
       <c r="H129" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I129" s="27">
-        <v>10.9</v>
+      <c r="I129" s="36">
+        <v>43.6</v>
       </c>
       <c r="J129" s="25" t="s">
         <v>377</v>
@@ -10364,11 +10412,11 @@
       </c>
       <c r="N129" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O129" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P129" s="8"/>
       <c r="Q129" s="50">
@@ -10405,8 +10453,8 @@
       <c r="H130" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I130" s="27">
-        <v>10.9</v>
+      <c r="I130" s="36">
+        <v>43.6</v>
       </c>
       <c r="J130" s="25" t="s">
         <v>377</v>
@@ -10422,11 +10470,11 @@
       </c>
       <c r="N130" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O130" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P130" s="8"/>
       <c r="Q130" s="50">
@@ -10463,8 +10511,8 @@
       <c r="H131" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I131" s="27">
-        <v>10.9</v>
+      <c r="I131" s="36">
+        <v>43.6</v>
       </c>
       <c r="J131" s="25" t="s">
         <v>377</v>
@@ -10480,11 +10528,11 @@
       </c>
       <c r="N131" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O131" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P131" s="8"/>
       <c r="Q131" s="50">
@@ -10521,8 +10569,8 @@
       <c r="H132" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I132" s="27">
-        <v>10.9</v>
+      <c r="I132" s="36">
+        <v>43.6</v>
       </c>
       <c r="J132" s="25" t="s">
         <v>377</v>
@@ -10538,11 +10586,11 @@
       </c>
       <c r="N132" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O132" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P132" s="8"/>
       <c r="Q132" s="50">
@@ -10579,8 +10627,8 @@
       <c r="H133" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I133" s="27">
-        <v>10.9</v>
+      <c r="I133" s="36">
+        <v>43.6</v>
       </c>
       <c r="J133" s="25" t="s">
         <v>377</v>
@@ -10596,11 +10644,11 @@
       </c>
       <c r="N133" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O133" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P133" s="8"/>
       <c r="Q133" s="50">
@@ -10637,8 +10685,8 @@
       <c r="H134" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I134" s="27">
-        <v>10.9</v>
+      <c r="I134" s="36">
+        <v>43.6</v>
       </c>
       <c r="J134" s="25" t="s">
         <v>377</v>
@@ -10654,11 +10702,11 @@
       </c>
       <c r="N134" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O134" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P134" s="8"/>
       <c r="Q134" s="50">
@@ -10695,8 +10743,8 @@
       <c r="H135" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I135" s="27">
-        <v>10.9</v>
+      <c r="I135" s="36">
+        <v>43.6</v>
       </c>
       <c r="J135" s="25" t="s">
         <v>377</v>
@@ -10712,11 +10760,11 @@
       </c>
       <c r="N135" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O135" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P135" s="8"/>
       <c r="Q135" s="50">
@@ -10753,8 +10801,8 @@
       <c r="H136" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I136" s="27">
-        <v>10.9</v>
+      <c r="I136" s="36">
+        <v>43.6</v>
       </c>
       <c r="J136" s="25" t="s">
         <v>377</v>
@@ -10770,11 +10818,11 @@
       </c>
       <c r="N136" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O136" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P136" s="8"/>
       <c r="Q136" s="50">
@@ -10811,8 +10859,8 @@
       <c r="H137" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I137" s="27">
-        <v>10.9</v>
+      <c r="I137" s="36">
+        <v>43.6</v>
       </c>
       <c r="J137" s="25" t="s">
         <v>377</v>
@@ -10828,11 +10876,11 @@
       </c>
       <c r="N137" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O137" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P137" s="8"/>
       <c r="Q137" s="50">
@@ -10927,8 +10975,8 @@
       <c r="H139" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I139" s="27">
-        <v>10.9</v>
+      <c r="I139" s="36">
+        <v>43.6</v>
       </c>
       <c r="J139" s="25" t="s">
         <v>377</v>
@@ -10944,11 +10992,11 @@
       </c>
       <c r="N139" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O139" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P139" s="8"/>
       <c r="Q139" s="50">
@@ -10985,8 +11033,8 @@
       <c r="H140" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I140" s="27">
-        <v>10.9</v>
+      <c r="I140" s="36">
+        <v>43.6</v>
       </c>
       <c r="J140" s="25" t="s">
         <v>377</v>
@@ -11002,11 +11050,11 @@
       </c>
       <c r="N140" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O140" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P140" s="8"/>
       <c r="Q140" s="50">
@@ -11043,8 +11091,8 @@
       <c r="H141" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I141" s="27">
-        <v>10.9</v>
+      <c r="I141" s="36">
+        <v>43.6</v>
       </c>
       <c r="J141" s="25" t="s">
         <v>377</v>
@@ -11060,11 +11108,11 @@
       </c>
       <c r="N141" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O141" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P141" s="8"/>
       <c r="Q141" s="50">
@@ -11101,8 +11149,8 @@
       <c r="H142" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I142" s="27">
-        <v>10.9</v>
+      <c r="I142" s="36">
+        <v>43.6</v>
       </c>
       <c r="J142" s="25" t="s">
         <v>377</v>
@@ -11118,11 +11166,11 @@
       </c>
       <c r="N142" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O142" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P142" s="8"/>
       <c r="Q142" s="50">
@@ -11159,8 +11207,8 @@
       <c r="H143" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I143" s="27">
-        <v>10.9</v>
+      <c r="I143" s="36">
+        <v>43.6</v>
       </c>
       <c r="J143" s="25" t="s">
         <v>377</v>
@@ -11176,11 +11224,11 @@
       </c>
       <c r="N143" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O143" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P143" s="8"/>
       <c r="Q143" s="50">
@@ -11217,8 +11265,8 @@
       <c r="H144" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I144" s="27">
-        <v>10.9</v>
+      <c r="I144" s="36">
+        <v>43.6</v>
       </c>
       <c r="J144" s="25" t="s">
         <v>377</v>
@@ -11234,11 +11282,11 @@
       </c>
       <c r="N144" s="30">
         <f t="shared" si="4"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O144" s="30">
         <f t="shared" si="5"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P144" s="8"/>
       <c r="Q144" s="50">
@@ -11275,8 +11323,8 @@
       <c r="H145" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I145" s="27">
-        <v>10.9</v>
+      <c r="I145" s="36">
+        <v>43.6</v>
       </c>
       <c r="J145" s="25" t="s">
         <v>377</v>
@@ -11292,11 +11340,11 @@
       </c>
       <c r="N145" s="30">
         <f t="shared" ref="N145:N208" si="8">I145*(1-M145)</f>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O145" s="30">
         <f t="shared" ref="O145:O208" si="9">N145*(1+J145)</f>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P145" s="8"/>
       <c r="Q145" s="50">
@@ -11333,8 +11381,8 @@
       <c r="H146" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I146" s="27">
-        <v>10.9</v>
+      <c r="I146" s="36">
+        <v>43.6</v>
       </c>
       <c r="J146" s="25" t="s">
         <v>377</v>
@@ -11350,11 +11398,11 @@
       </c>
       <c r="N146" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O146" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P146" s="8"/>
       <c r="Q146" s="50">
@@ -11391,8 +11439,8 @@
       <c r="H147" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I147" s="27">
-        <v>10.9</v>
+      <c r="I147" s="36">
+        <v>43.6</v>
       </c>
       <c r="J147" s="25" t="s">
         <v>377</v>
@@ -11408,11 +11456,11 @@
       </c>
       <c r="N147" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O147" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P147" s="8"/>
       <c r="Q147" s="50">
@@ -11449,8 +11497,8 @@
       <c r="H148" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I148" s="27">
-        <v>10.9</v>
+      <c r="I148" s="36">
+        <v>43.6</v>
       </c>
       <c r="J148" s="25" t="s">
         <v>377</v>
@@ -11466,11 +11514,11 @@
       </c>
       <c r="N148" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O148" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P148" s="8"/>
       <c r="Q148" s="50">
@@ -11507,8 +11555,8 @@
       <c r="H149" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I149" s="27">
-        <v>10.9</v>
+      <c r="I149" s="36">
+        <v>43.6</v>
       </c>
       <c r="J149" s="25" t="s">
         <v>377</v>
@@ -11524,11 +11572,11 @@
       </c>
       <c r="N149" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O149" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P149" s="8"/>
       <c r="Q149" s="50">
@@ -11565,8 +11613,8 @@
       <c r="H150" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I150" s="27">
-        <v>10.9</v>
+      <c r="I150" s="36">
+        <v>43.6</v>
       </c>
       <c r="J150" s="25" t="s">
         <v>377</v>
@@ -11582,11 +11630,11 @@
       </c>
       <c r="N150" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O150" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P150" s="8"/>
       <c r="Q150" s="50">
@@ -11623,8 +11671,8 @@
       <c r="H151" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I151" s="27">
-        <v>10.9</v>
+      <c r="I151" s="36">
+        <v>43.6</v>
       </c>
       <c r="J151" s="25" t="s">
         <v>377</v>
@@ -11640,11 +11688,11 @@
       </c>
       <c r="N151" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O151" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P151" s="8"/>
       <c r="Q151" s="50">
@@ -11681,8 +11729,8 @@
       <c r="H152" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I152" s="27">
-        <v>10.9</v>
+      <c r="I152" s="36">
+        <v>43.6</v>
       </c>
       <c r="J152" s="25" t="s">
         <v>377</v>
@@ -11698,11 +11746,11 @@
       </c>
       <c r="N152" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O152" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P152" s="8"/>
       <c r="Q152" s="50">
@@ -11739,8 +11787,8 @@
       <c r="H153" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I153" s="27">
-        <v>10.9</v>
+      <c r="I153" s="36">
+        <v>43.6</v>
       </c>
       <c r="J153" s="25" t="s">
         <v>377</v>
@@ -11756,11 +11804,11 @@
       </c>
       <c r="N153" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O153" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P153" s="8"/>
       <c r="Q153" s="50">
@@ -11797,8 +11845,8 @@
       <c r="H154" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I154" s="27">
-        <v>10.9</v>
+      <c r="I154" s="36">
+        <v>43.6</v>
       </c>
       <c r="J154" s="25" t="s">
         <v>377</v>
@@ -11814,11 +11862,11 @@
       </c>
       <c r="N154" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O154" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P154" s="8"/>
       <c r="Q154" s="50">
@@ -11855,8 +11903,8 @@
       <c r="H155" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I155" s="27">
-        <v>10.9</v>
+      <c r="I155" s="36">
+        <v>43.6</v>
       </c>
       <c r="J155" s="25" t="s">
         <v>377</v>
@@ -11872,11 +11920,11 @@
       </c>
       <c r="N155" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O155" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P155" s="8"/>
       <c r="Q155" s="50">
@@ -11913,8 +11961,8 @@
       <c r="H156" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I156" s="27">
-        <v>10.9</v>
+      <c r="I156" s="36">
+        <v>43.6</v>
       </c>
       <c r="J156" s="25" t="s">
         <v>377</v>
@@ -11930,11 +11978,11 @@
       </c>
       <c r="N156" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O156" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P156" s="8"/>
       <c r="Q156" s="50">
@@ -11971,8 +12019,8 @@
       <c r="H157" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I157" s="27">
-        <v>10.9</v>
+      <c r="I157" s="36">
+        <v>43.6</v>
       </c>
       <c r="J157" s="25" t="s">
         <v>377</v>
@@ -11988,11 +12036,11 @@
       </c>
       <c r="N157" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O157" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P157" s="8"/>
       <c r="Q157" s="50">
@@ -12029,8 +12077,8 @@
       <c r="H158" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I158" s="27">
-        <v>10.9</v>
+      <c r="I158" s="36">
+        <v>43.6</v>
       </c>
       <c r="J158" s="25" t="s">
         <v>377</v>
@@ -12046,11 +12094,11 @@
       </c>
       <c r="N158" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O158" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P158" s="8"/>
       <c r="Q158" s="50">
@@ -12087,8 +12135,8 @@
       <c r="H159" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I159" s="27">
-        <v>10.9</v>
+      <c r="I159" s="36">
+        <v>43.6</v>
       </c>
       <c r="J159" s="25" t="s">
         <v>377</v>
@@ -12104,11 +12152,11 @@
       </c>
       <c r="N159" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O159" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P159" s="8"/>
       <c r="Q159" s="50">
@@ -12145,8 +12193,8 @@
       <c r="H160" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I160" s="27">
-        <v>10.9</v>
+      <c r="I160" s="36">
+        <v>43.6</v>
       </c>
       <c r="J160" s="25" t="s">
         <v>377</v>
@@ -12162,11 +12210,11 @@
       </c>
       <c r="N160" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O160" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P160" s="8"/>
       <c r="Q160" s="50">
@@ -12203,8 +12251,8 @@
       <c r="H161" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I161" s="27">
-        <v>10.9</v>
+      <c r="I161" s="36">
+        <v>43.6</v>
       </c>
       <c r="J161" s="25" t="s">
         <v>377</v>
@@ -12220,11 +12268,11 @@
       </c>
       <c r="N161" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O161" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P161" s="8"/>
       <c r="Q161" s="50">
@@ -12261,8 +12309,8 @@
       <c r="H162" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I162" s="27">
-        <v>10.9</v>
+      <c r="I162" s="36">
+        <v>43.6</v>
       </c>
       <c r="J162" s="25" t="s">
         <v>377</v>
@@ -12278,11 +12326,11 @@
       </c>
       <c r="N162" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O162" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P162" s="8"/>
       <c r="Q162" s="50">
@@ -12377,8 +12425,8 @@
       <c r="H164" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I164" s="27">
-        <v>10.9</v>
+      <c r="I164" s="36">
+        <v>43.6</v>
       </c>
       <c r="J164" s="25" t="s">
         <v>377</v>
@@ -12394,11 +12442,11 @@
       </c>
       <c r="N164" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O164" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P164" s="8"/>
       <c r="Q164" s="50">
@@ -12435,8 +12483,8 @@
       <c r="H165" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I165" s="27">
-        <v>10.9</v>
+      <c r="I165" s="36">
+        <v>43.6</v>
       </c>
       <c r="J165" s="25" t="s">
         <v>377</v>
@@ -12452,11 +12500,11 @@
       </c>
       <c r="N165" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O165" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P165" s="8"/>
       <c r="Q165" s="50">
@@ -12493,8 +12541,8 @@
       <c r="H166" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I166" s="27">
-        <v>10.9</v>
+      <c r="I166" s="36">
+        <v>43.6</v>
       </c>
       <c r="J166" s="25" t="s">
         <v>377</v>
@@ -12510,11 +12558,11 @@
       </c>
       <c r="N166" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O166" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P166" s="8"/>
       <c r="Q166" s="50">
@@ -12551,8 +12599,8 @@
       <c r="H167" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I167" s="27">
-        <v>10.9</v>
+      <c r="I167" s="36">
+        <v>43.6</v>
       </c>
       <c r="J167" s="25" t="s">
         <v>377</v>
@@ -12568,11 +12616,11 @@
       </c>
       <c r="N167" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O167" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P167" s="8"/>
       <c r="Q167" s="50">
@@ -12609,8 +12657,8 @@
       <c r="H168" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I168" s="27">
-        <v>10.9</v>
+      <c r="I168" s="36">
+        <v>43.6</v>
       </c>
       <c r="J168" s="25" t="s">
         <v>377</v>
@@ -12626,11 +12674,11 @@
       </c>
       <c r="N168" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O168" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P168" s="8"/>
       <c r="Q168" s="50">
@@ -12667,8 +12715,8 @@
       <c r="H169" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I169" s="27">
-        <v>10.9</v>
+      <c r="I169" s="36">
+        <v>43.6</v>
       </c>
       <c r="J169" s="25" t="s">
         <v>377</v>
@@ -12684,11 +12732,11 @@
       </c>
       <c r="N169" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O169" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P169" s="8"/>
       <c r="Q169" s="50">
@@ -12783,8 +12831,8 @@
       <c r="H171" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I171" s="27">
-        <v>10.9</v>
+      <c r="I171" s="36">
+        <v>43.6</v>
       </c>
       <c r="J171" s="25" t="s">
         <v>377</v>
@@ -12800,11 +12848,11 @@
       </c>
       <c r="N171" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O171" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P171" s="8"/>
       <c r="Q171" s="50">
@@ -12841,8 +12889,8 @@
       <c r="H172" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I172" s="27">
-        <v>10.9</v>
+      <c r="I172" s="36">
+        <v>43.6</v>
       </c>
       <c r="J172" s="25" t="s">
         <v>377</v>
@@ -12858,11 +12906,11 @@
       </c>
       <c r="N172" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O172" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P172" s="8"/>
       <c r="Q172" s="50">
@@ -12899,8 +12947,8 @@
       <c r="H173" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I173" s="27">
-        <v>10.9</v>
+      <c r="I173" s="36">
+        <v>43.6</v>
       </c>
       <c r="J173" s="25" t="s">
         <v>377</v>
@@ -12916,11 +12964,11 @@
       </c>
       <c r="N173" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O173" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P173" s="8"/>
       <c r="Q173" s="50">
@@ -12957,8 +13005,8 @@
       <c r="H174" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I174" s="27">
-        <v>10.9</v>
+      <c r="I174" s="36">
+        <v>43.6</v>
       </c>
       <c r="J174" s="25" t="s">
         <v>377</v>
@@ -12974,11 +13022,11 @@
       </c>
       <c r="N174" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O174" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P174" s="8"/>
       <c r="Q174" s="50">
@@ -13015,8 +13063,8 @@
       <c r="H175" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I175" s="27">
-        <v>10.9</v>
+      <c r="I175" s="36">
+        <v>43.6</v>
       </c>
       <c r="J175" s="25" t="s">
         <v>377</v>
@@ -13032,11 +13080,11 @@
       </c>
       <c r="N175" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O175" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P175" s="8"/>
       <c r="Q175" s="50">
@@ -13073,8 +13121,8 @@
       <c r="H176" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I176" s="27">
-        <v>10.9</v>
+      <c r="I176" s="36">
+        <v>43.6</v>
       </c>
       <c r="J176" s="25" t="s">
         <v>377</v>
@@ -13090,11 +13138,11 @@
       </c>
       <c r="N176" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O176" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P176" s="8"/>
       <c r="Q176" s="50">
@@ -13189,8 +13237,8 @@
       <c r="H178" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I178" s="27">
-        <v>10.9</v>
+      <c r="I178" s="36">
+        <v>43.6</v>
       </c>
       <c r="J178" s="25" t="s">
         <v>377</v>
@@ -13206,11 +13254,11 @@
       </c>
       <c r="N178" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O178" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P178" s="8"/>
       <c r="Q178" s="50">
@@ -13247,8 +13295,8 @@
       <c r="H179" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I179" s="27">
-        <v>10.9</v>
+      <c r="I179" s="36">
+        <v>43.6</v>
       </c>
       <c r="J179" s="25" t="s">
         <v>377</v>
@@ -13264,11 +13312,11 @@
       </c>
       <c r="N179" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O179" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P179" s="8"/>
       <c r="Q179" s="50">
@@ -13305,8 +13353,8 @@
       <c r="H180" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I180" s="27">
-        <v>10.9</v>
+      <c r="I180" s="36">
+        <v>43.6</v>
       </c>
       <c r="J180" s="25" t="s">
         <v>377</v>
@@ -13322,11 +13370,11 @@
       </c>
       <c r="N180" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O180" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P180" s="8"/>
       <c r="Q180" s="50">
@@ -13363,8 +13411,8 @@
       <c r="H181" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I181" s="27">
-        <v>10.9</v>
+      <c r="I181" s="36">
+        <v>43.6</v>
       </c>
       <c r="J181" s="25" t="s">
         <v>377</v>
@@ -13380,11 +13428,11 @@
       </c>
       <c r="N181" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O181" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P181" s="8"/>
       <c r="Q181" s="50">
@@ -13421,8 +13469,8 @@
       <c r="H182" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I182" s="27">
-        <v>10.9</v>
+      <c r="I182" s="36">
+        <v>43.6</v>
       </c>
       <c r="J182" s="25" t="s">
         <v>377</v>
@@ -13438,11 +13486,11 @@
       </c>
       <c r="N182" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O182" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P182" s="8"/>
       <c r="Q182" s="50">
@@ -13479,8 +13527,8 @@
       <c r="H183" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I183" s="27">
-        <v>10.9</v>
+      <c r="I183" s="36">
+        <v>43.6</v>
       </c>
       <c r="J183" s="25" t="s">
         <v>377</v>
@@ -13496,11 +13544,11 @@
       </c>
       <c r="N183" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O183" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P183" s="8"/>
       <c r="Q183" s="50">
@@ -13595,8 +13643,8 @@
       <c r="H185" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I185" s="27">
-        <v>10.9</v>
+      <c r="I185" s="36">
+        <v>43.6</v>
       </c>
       <c r="J185" s="25" t="s">
         <v>377</v>
@@ -13612,11 +13660,11 @@
       </c>
       <c r="N185" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O185" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P185" s="8"/>
       <c r="Q185" s="50">
@@ -13653,8 +13701,8 @@
       <c r="H186" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I186" s="27">
-        <v>10.9</v>
+      <c r="I186" s="36">
+        <v>43.6</v>
       </c>
       <c r="J186" s="25" t="s">
         <v>377</v>
@@ -13670,11 +13718,11 @@
       </c>
       <c r="N186" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O186" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P186" s="8"/>
       <c r="Q186" s="50">
@@ -13711,8 +13759,8 @@
       <c r="H187" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I187" s="27">
-        <v>10.9</v>
+      <c r="I187" s="36">
+        <v>43.6</v>
       </c>
       <c r="J187" s="25" t="s">
         <v>377</v>
@@ -13728,11 +13776,11 @@
       </c>
       <c r="N187" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O187" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P187" s="8"/>
       <c r="Q187" s="50">
@@ -13769,8 +13817,8 @@
       <c r="H188" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I188" s="27">
-        <v>10.9</v>
+      <c r="I188" s="36">
+        <v>43.6</v>
       </c>
       <c r="J188" s="25" t="s">
         <v>377</v>
@@ -13786,11 +13834,11 @@
       </c>
       <c r="N188" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O188" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P188" s="8"/>
       <c r="Q188" s="50">
@@ -13827,8 +13875,8 @@
       <c r="H189" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I189" s="27">
-        <v>10.9</v>
+      <c r="I189" s="36">
+        <v>43.6</v>
       </c>
       <c r="J189" s="25" t="s">
         <v>377</v>
@@ -13844,11 +13892,11 @@
       </c>
       <c r="N189" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O189" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P189" s="8"/>
       <c r="Q189" s="50">
@@ -13885,8 +13933,8 @@
       <c r="H190" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I190" s="27">
-        <v>10.9</v>
+      <c r="I190" s="36">
+        <v>43.6</v>
       </c>
       <c r="J190" s="25" t="s">
         <v>377</v>
@@ -13902,11 +13950,11 @@
       </c>
       <c r="N190" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O190" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P190" s="8"/>
       <c r="Q190" s="50">
@@ -14001,8 +14049,8 @@
       <c r="H192" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I192" s="27">
-        <v>10.9</v>
+      <c r="I192" s="36">
+        <v>43.6</v>
       </c>
       <c r="J192" s="25" t="s">
         <v>377</v>
@@ -14018,11 +14066,11 @@
       </c>
       <c r="N192" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O192" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P192" s="8"/>
       <c r="Q192" s="50">
@@ -14059,8 +14107,8 @@
       <c r="H193" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I193" s="27">
-        <v>10.9</v>
+      <c r="I193" s="36">
+        <v>43.6</v>
       </c>
       <c r="J193" s="25" t="s">
         <v>377</v>
@@ -14076,11 +14124,11 @@
       </c>
       <c r="N193" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O193" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P193" s="8"/>
       <c r="Q193" s="50">
@@ -14117,8 +14165,8 @@
       <c r="H194" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I194" s="27">
-        <v>10.9</v>
+      <c r="I194" s="36">
+        <v>43.6</v>
       </c>
       <c r="J194" s="25" t="s">
         <v>377</v>
@@ -14134,11 +14182,11 @@
       </c>
       <c r="N194" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O194" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P194" s="8"/>
       <c r="Q194" s="50">
@@ -14175,8 +14223,8 @@
       <c r="H195" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I195" s="27">
-        <v>10.9</v>
+      <c r="I195" s="36">
+        <v>43.6</v>
       </c>
       <c r="J195" s="25" t="s">
         <v>377</v>
@@ -14192,11 +14240,11 @@
       </c>
       <c r="N195" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O195" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P195" s="8"/>
       <c r="Q195" s="50">
@@ -14233,8 +14281,8 @@
       <c r="H196" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I196" s="27">
-        <v>10.9</v>
+      <c r="I196" s="36">
+        <v>43.6</v>
       </c>
       <c r="J196" s="25" t="s">
         <v>377</v>
@@ -14250,11 +14298,11 @@
       </c>
       <c r="N196" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O196" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P196" s="8"/>
       <c r="Q196" s="50">
@@ -14291,8 +14339,8 @@
       <c r="H197" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I197" s="27">
-        <v>10.9</v>
+      <c r="I197" s="36">
+        <v>43.6</v>
       </c>
       <c r="J197" s="25" t="s">
         <v>377</v>
@@ -14308,11 +14356,11 @@
       </c>
       <c r="N197" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O197" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P197" s="8"/>
       <c r="Q197" s="50">
@@ -14407,8 +14455,8 @@
       <c r="H199" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I199" s="27">
-        <v>10.9</v>
+      <c r="I199" s="36">
+        <v>43.6</v>
       </c>
       <c r="J199" s="25" t="s">
         <v>377</v>
@@ -14424,11 +14472,11 @@
       </c>
       <c r="N199" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O199" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P199" s="8"/>
       <c r="Q199" s="50">
@@ -14465,8 +14513,8 @@
       <c r="H200" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I200" s="27">
-        <v>10.9</v>
+      <c r="I200" s="36">
+        <v>43.6</v>
       </c>
       <c r="J200" s="25" t="s">
         <v>377</v>
@@ -14482,11 +14530,11 @@
       </c>
       <c r="N200" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O200" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P200" s="8"/>
       <c r="Q200" s="50">
@@ -14523,8 +14571,8 @@
       <c r="H201" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I201" s="27">
-        <v>10.9</v>
+      <c r="I201" s="36">
+        <v>43.6</v>
       </c>
       <c r="J201" s="25" t="s">
         <v>377</v>
@@ -14540,11 +14588,11 @@
       </c>
       <c r="N201" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O201" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P201" s="8"/>
       <c r="Q201" s="50">
@@ -14581,8 +14629,8 @@
       <c r="H202" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I202" s="27">
-        <v>10.9</v>
+      <c r="I202" s="36">
+        <v>43.6</v>
       </c>
       <c r="J202" s="25" t="s">
         <v>377</v>
@@ -14598,11 +14646,11 @@
       </c>
       <c r="N202" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O202" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P202" s="8"/>
       <c r="Q202" s="50">
@@ -14639,8 +14687,8 @@
       <c r="H203" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I203" s="27">
-        <v>10.9</v>
+      <c r="I203" s="36">
+        <v>43.6</v>
       </c>
       <c r="J203" s="25" t="s">
         <v>377</v>
@@ -14656,11 +14704,11 @@
       </c>
       <c r="N203" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O203" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P203" s="8"/>
       <c r="Q203" s="50">
@@ -14697,8 +14745,8 @@
       <c r="H204" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I204" s="27">
-        <v>10.9</v>
+      <c r="I204" s="36">
+        <v>43.6</v>
       </c>
       <c r="J204" s="25" t="s">
         <v>377</v>
@@ -14714,11 +14762,11 @@
       </c>
       <c r="N204" s="30">
         <f t="shared" si="8"/>
-        <v>4.3600000000000003</v>
+        <v>17.440000000000001</v>
       </c>
       <c r="O204" s="30">
         <f t="shared" si="9"/>
-        <v>4.5344000000000007</v>
+        <v>18.137600000000003</v>
       </c>
       <c r="P204" s="8"/>
       <c r="Q204" s="50">
@@ -14811,8 +14859,8 @@
       <c r="H206" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I206" s="27">
-        <v>10.9</v>
+      <c r="I206" s="36">
+        <v>43.6</v>
       </c>
       <c r="J206" s="25" t="s">
         <v>377</v>
@@ -14826,11 +14874,11 @@
       </c>
       <c r="N206" s="30">
         <f t="shared" si="8"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O206" s="30">
         <f t="shared" si="9"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P206" s="8"/>
       <c r="Q206" s="50">
@@ -14867,8 +14915,8 @@
       <c r="H207" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I207" s="27">
-        <v>10.9</v>
+      <c r="I207" s="36">
+        <v>43.6</v>
       </c>
       <c r="J207" s="25" t="s">
         <v>377</v>
@@ -14882,11 +14930,11 @@
       </c>
       <c r="N207" s="30">
         <f t="shared" si="8"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O207" s="30">
         <f t="shared" si="9"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P207" s="8"/>
       <c r="Q207" s="50">
@@ -14923,8 +14971,8 @@
       <c r="H208" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I208" s="27">
-        <v>10.9</v>
+      <c r="I208" s="36">
+        <v>43.6</v>
       </c>
       <c r="J208" s="25" t="s">
         <v>377</v>
@@ -14938,11 +14986,11 @@
       </c>
       <c r="N208" s="30">
         <f t="shared" si="8"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O208" s="30">
         <f t="shared" si="9"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P208" s="8"/>
       <c r="Q208" s="50">
@@ -14979,8 +15027,8 @@
       <c r="H209" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I209" s="27">
-        <v>10.9</v>
+      <c r="I209" s="36">
+        <v>43.6</v>
       </c>
       <c r="J209" s="25" t="s">
         <v>377</v>
@@ -14994,11 +15042,11 @@
       </c>
       <c r="N209" s="30">
         <f t="shared" ref="N209:N272" si="12">I209*(1-M209)</f>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O209" s="30">
         <f t="shared" ref="O209:O272" si="13">N209*(1+J209)</f>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P209" s="8"/>
       <c r="Q209" s="50">
@@ -15035,8 +15083,8 @@
       <c r="H210" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I210" s="27">
-        <v>10.9</v>
+      <c r="I210" s="36">
+        <v>43.6</v>
       </c>
       <c r="J210" s="25" t="s">
         <v>377</v>
@@ -15050,11 +15098,11 @@
       </c>
       <c r="N210" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O210" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P210" s="8"/>
       <c r="Q210" s="50">
@@ -15091,8 +15139,8 @@
       <c r="H211" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I211" s="27">
-        <v>10.9</v>
+      <c r="I211" s="36">
+        <v>43.6</v>
       </c>
       <c r="J211" s="25" t="s">
         <v>377</v>
@@ -15106,11 +15154,11 @@
       </c>
       <c r="N211" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O211" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P211" s="8"/>
       <c r="Q211" s="50">
@@ -15203,8 +15251,8 @@
       <c r="H213" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I213" s="27">
-        <v>10.9</v>
+      <c r="I213" s="36">
+        <v>43.6</v>
       </c>
       <c r="J213" s="25" t="s">
         <v>377</v>
@@ -15218,11 +15266,11 @@
       </c>
       <c r="N213" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O213" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P213" s="8"/>
       <c r="Q213" s="50">
@@ -15259,8 +15307,8 @@
       <c r="H214" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I214" s="27">
-        <v>10.9</v>
+      <c r="I214" s="36">
+        <v>43.6</v>
       </c>
       <c r="J214" s="25" t="s">
         <v>377</v>
@@ -15274,11 +15322,11 @@
       </c>
       <c r="N214" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O214" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P214" s="8"/>
       <c r="Q214" s="50">
@@ -15315,8 +15363,8 @@
       <c r="H215" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I215" s="27">
-        <v>10.9</v>
+      <c r="I215" s="36">
+        <v>43.6</v>
       </c>
       <c r="J215" s="25" t="s">
         <v>377</v>
@@ -15330,11 +15378,11 @@
       </c>
       <c r="N215" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O215" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P215" s="8"/>
       <c r="Q215" s="50">
@@ -15371,8 +15419,8 @@
       <c r="H216" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I216" s="27">
-        <v>10.9</v>
+      <c r="I216" s="36">
+        <v>43.6</v>
       </c>
       <c r="J216" s="25" t="s">
         <v>377</v>
@@ -15386,11 +15434,11 @@
       </c>
       <c r="N216" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O216" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P216" s="8"/>
       <c r="Q216" s="50">
@@ -15427,8 +15475,8 @@
       <c r="H217" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I217" s="27">
-        <v>10.9</v>
+      <c r="I217" s="36">
+        <v>43.6</v>
       </c>
       <c r="J217" s="25" t="s">
         <v>377</v>
@@ -15442,11 +15490,11 @@
       </c>
       <c r="N217" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O217" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P217" s="8"/>
       <c r="Q217" s="50">
@@ -15483,8 +15531,8 @@
       <c r="H218" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I218" s="27">
-        <v>10.9</v>
+      <c r="I218" s="36">
+        <v>43.6</v>
       </c>
       <c r="J218" s="25" t="s">
         <v>377</v>
@@ -15498,11 +15546,11 @@
       </c>
       <c r="N218" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O218" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P218" s="8"/>
       <c r="Q218" s="50">
@@ -15595,8 +15643,8 @@
       <c r="H220" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I220" s="27">
-        <v>10.9</v>
+      <c r="I220" s="36">
+        <v>43.6</v>
       </c>
       <c r="J220" s="25" t="s">
         <v>377</v>
@@ -15610,11 +15658,11 @@
       </c>
       <c r="N220" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O220" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P220" s="8"/>
       <c r="Q220" s="50">
@@ -15651,8 +15699,8 @@
       <c r="H221" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I221" s="27">
-        <v>10.9</v>
+      <c r="I221" s="36">
+        <v>43.6</v>
       </c>
       <c r="J221" s="25" t="s">
         <v>377</v>
@@ -15666,11 +15714,11 @@
       </c>
       <c r="N221" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O221" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P221" s="8"/>
       <c r="Q221" s="50">
@@ -15707,8 +15755,8 @@
       <c r="H222" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I222" s="27">
-        <v>10.9</v>
+      <c r="I222" s="36">
+        <v>43.6</v>
       </c>
       <c r="J222" s="25" t="s">
         <v>377</v>
@@ -15722,11 +15770,11 @@
       </c>
       <c r="N222" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O222" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P222" s="8"/>
       <c r="Q222" s="50">
@@ -15763,8 +15811,8 @@
       <c r="H223" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I223" s="27">
-        <v>10.9</v>
+      <c r="I223" s="36">
+        <v>43.6</v>
       </c>
       <c r="J223" s="25" t="s">
         <v>377</v>
@@ -15778,11 +15826,11 @@
       </c>
       <c r="N223" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O223" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P223" s="8"/>
       <c r="Q223" s="50">
@@ -15819,8 +15867,8 @@
       <c r="H224" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I224" s="27">
-        <v>10.9</v>
+      <c r="I224" s="36">
+        <v>43.6</v>
       </c>
       <c r="J224" s="25" t="s">
         <v>377</v>
@@ -15834,11 +15882,11 @@
       </c>
       <c r="N224" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O224" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P224" s="8"/>
       <c r="Q224" s="50">
@@ -15875,8 +15923,8 @@
       <c r="H225" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I225" s="27">
-        <v>10.9</v>
+      <c r="I225" s="36">
+        <v>43.6</v>
       </c>
       <c r="J225" s="25" t="s">
         <v>377</v>
@@ -15890,11 +15938,11 @@
       </c>
       <c r="N225" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O225" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P225" s="8"/>
       <c r="Q225" s="50">
@@ -15987,8 +16035,8 @@
       <c r="H227" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I227" s="27">
-        <v>10.9</v>
+      <c r="I227" s="36">
+        <v>43.6</v>
       </c>
       <c r="J227" s="25" t="s">
         <v>377</v>
@@ -16002,11 +16050,11 @@
       </c>
       <c r="N227" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O227" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P227" s="8"/>
       <c r="Q227" s="50">
@@ -16043,8 +16091,8 @@
       <c r="H228" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I228" s="27">
-        <v>10.9</v>
+      <c r="I228" s="36">
+        <v>43.6</v>
       </c>
       <c r="J228" s="25" t="s">
         <v>377</v>
@@ -16058,11 +16106,11 @@
       </c>
       <c r="N228" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O228" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P228" s="8"/>
       <c r="Q228" s="50">
@@ -16099,8 +16147,8 @@
       <c r="H229" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I229" s="27">
-        <v>10.9</v>
+      <c r="I229" s="36">
+        <v>43.6</v>
       </c>
       <c r="J229" s="25" t="s">
         <v>377</v>
@@ -16114,11 +16162,11 @@
       </c>
       <c r="N229" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O229" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P229" s="8"/>
       <c r="Q229" s="50">
@@ -16155,8 +16203,8 @@
       <c r="H230" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I230" s="27">
-        <v>10.9</v>
+      <c r="I230" s="36">
+        <v>43.6</v>
       </c>
       <c r="J230" s="25" t="s">
         <v>377</v>
@@ -16170,11 +16218,11 @@
       </c>
       <c r="N230" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O230" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P230" s="8"/>
       <c r="Q230" s="50">
@@ -16211,8 +16259,8 @@
       <c r="H231" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I231" s="27">
-        <v>10.9</v>
+      <c r="I231" s="36">
+        <v>43.6</v>
       </c>
       <c r="J231" s="25" t="s">
         <v>377</v>
@@ -16226,11 +16274,11 @@
       </c>
       <c r="N231" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O231" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P231" s="8"/>
       <c r="Q231" s="50">
@@ -16267,8 +16315,8 @@
       <c r="H232" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I232" s="27">
-        <v>10.9</v>
+      <c r="I232" s="36">
+        <v>43.6</v>
       </c>
       <c r="J232" s="25" t="s">
         <v>377</v>
@@ -16282,11 +16330,11 @@
       </c>
       <c r="N232" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O232" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P232" s="8"/>
       <c r="Q232" s="50">
@@ -16379,8 +16427,8 @@
       <c r="H234" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I234" s="27">
-        <v>10.9</v>
+      <c r="I234" s="36">
+        <v>43.6</v>
       </c>
       <c r="J234" s="25" t="s">
         <v>377</v>
@@ -16394,11 +16442,11 @@
       </c>
       <c r="N234" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O234" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P234" s="8"/>
       <c r="Q234" s="50">
@@ -16435,8 +16483,8 @@
       <c r="H235" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I235" s="27">
-        <v>10.9</v>
+      <c r="I235" s="36">
+        <v>43.6</v>
       </c>
       <c r="J235" s="25" t="s">
         <v>377</v>
@@ -16450,11 +16498,11 @@
       </c>
       <c r="N235" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O235" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P235" s="8"/>
       <c r="Q235" s="50">
@@ -16491,8 +16539,8 @@
       <c r="H236" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I236" s="27">
-        <v>10.9</v>
+      <c r="I236" s="36">
+        <v>43.6</v>
       </c>
       <c r="J236" s="25" t="s">
         <v>377</v>
@@ -16506,11 +16554,11 @@
       </c>
       <c r="N236" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O236" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P236" s="8"/>
       <c r="Q236" s="50">
@@ -16547,8 +16595,8 @@
       <c r="H237" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I237" s="27">
-        <v>10.9</v>
+      <c r="I237" s="36">
+        <v>43.6</v>
       </c>
       <c r="J237" s="25" t="s">
         <v>377</v>
@@ -16562,11 +16610,11 @@
       </c>
       <c r="N237" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O237" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P237" s="8"/>
       <c r="Q237" s="50">
@@ -16603,8 +16651,8 @@
       <c r="H238" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I238" s="27">
-        <v>10.9</v>
+      <c r="I238" s="36">
+        <v>43.6</v>
       </c>
       <c r="J238" s="25" t="s">
         <v>377</v>
@@ -16618,11 +16666,11 @@
       </c>
       <c r="N238" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O238" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P238" s="8"/>
       <c r="Q238" s="50">
@@ -16659,8 +16707,8 @@
       <c r="H239" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I239" s="27">
-        <v>10.9</v>
+      <c r="I239" s="36">
+        <v>43.6</v>
       </c>
       <c r="J239" s="25" t="s">
         <v>377</v>
@@ -16674,11 +16722,11 @@
       </c>
       <c r="N239" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O239" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P239" s="8"/>
       <c r="Q239" s="50">
@@ -16771,8 +16819,8 @@
       <c r="H241" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I241" s="27">
-        <v>10.9</v>
+      <c r="I241" s="36">
+        <v>43.6</v>
       </c>
       <c r="J241" s="25" t="s">
         <v>377</v>
@@ -16786,11 +16834,11 @@
       </c>
       <c r="N241" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O241" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P241" s="8"/>
       <c r="Q241" s="50">
@@ -16827,8 +16875,8 @@
       <c r="H242" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I242" s="27">
-        <v>10.9</v>
+      <c r="I242" s="36">
+        <v>43.6</v>
       </c>
       <c r="J242" s="25" t="s">
         <v>377</v>
@@ -16842,11 +16890,11 @@
       </c>
       <c r="N242" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O242" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P242" s="8"/>
       <c r="Q242" s="50">
@@ -16883,8 +16931,8 @@
       <c r="H243" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I243" s="27">
-        <v>10.9</v>
+      <c r="I243" s="36">
+        <v>43.6</v>
       </c>
       <c r="J243" s="25" t="s">
         <v>377</v>
@@ -16898,11 +16946,11 @@
       </c>
       <c r="N243" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O243" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P243" s="8"/>
       <c r="Q243" s="50">
@@ -16939,8 +16987,8 @@
       <c r="H244" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I244" s="27">
-        <v>10.9</v>
+      <c r="I244" s="36">
+        <v>43.6</v>
       </c>
       <c r="J244" s="25" t="s">
         <v>377</v>
@@ -16954,11 +17002,11 @@
       </c>
       <c r="N244" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O244" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P244" s="8"/>
       <c r="Q244" s="50">
@@ -16995,8 +17043,8 @@
       <c r="H245" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I245" s="27">
-        <v>10.9</v>
+      <c r="I245" s="36">
+        <v>43.6</v>
       </c>
       <c r="J245" s="25" t="s">
         <v>377</v>
@@ -17010,11 +17058,11 @@
       </c>
       <c r="N245" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O245" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P245" s="8"/>
       <c r="Q245" s="50">
@@ -17051,8 +17099,8 @@
       <c r="H246" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I246" s="27">
-        <v>10.9</v>
+      <c r="I246" s="36">
+        <v>43.6</v>
       </c>
       <c r="J246" s="25" t="s">
         <v>377</v>
@@ -17066,11 +17114,11 @@
       </c>
       <c r="N246" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O246" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P246" s="8"/>
       <c r="Q246" s="50">
@@ -17163,8 +17211,8 @@
       <c r="H248" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I248" s="27">
-        <v>10.9</v>
+      <c r="I248" s="36">
+        <v>43.6</v>
       </c>
       <c r="J248" s="25" t="s">
         <v>377</v>
@@ -17178,11 +17226,11 @@
       </c>
       <c r="N248" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O248" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P248" s="8"/>
       <c r="Q248" s="50">
@@ -17219,8 +17267,8 @@
       <c r="H249" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I249" s="27">
-        <v>10.9</v>
+      <c r="I249" s="36">
+        <v>43.6</v>
       </c>
       <c r="J249" s="25" t="s">
         <v>377</v>
@@ -17234,11 +17282,11 @@
       </c>
       <c r="N249" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O249" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P249" s="8"/>
       <c r="Q249" s="50">
@@ -17275,8 +17323,8 @@
       <c r="H250" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I250" s="27">
-        <v>10.9</v>
+      <c r="I250" s="36">
+        <v>43.6</v>
       </c>
       <c r="J250" s="25" t="s">
         <v>377</v>
@@ -17290,11 +17338,11 @@
       </c>
       <c r="N250" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O250" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P250" s="8"/>
       <c r="Q250" s="50">
@@ -17331,8 +17379,8 @@
       <c r="H251" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I251" s="27">
-        <v>10.9</v>
+      <c r="I251" s="36">
+        <v>43.6</v>
       </c>
       <c r="J251" s="25" t="s">
         <v>377</v>
@@ -17346,11 +17394,11 @@
       </c>
       <c r="N251" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O251" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P251" s="8"/>
       <c r="Q251" s="50">
@@ -17387,8 +17435,8 @@
       <c r="H252" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I252" s="27">
-        <v>10.9</v>
+      <c r="I252" s="36">
+        <v>43.6</v>
       </c>
       <c r="J252" s="25" t="s">
         <v>377</v>
@@ -17402,11 +17450,11 @@
       </c>
       <c r="N252" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O252" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P252" s="8"/>
       <c r="Q252" s="50">
@@ -17443,8 +17491,8 @@
       <c r="H253" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I253" s="27">
-        <v>10.9</v>
+      <c r="I253" s="36">
+        <v>43.6</v>
       </c>
       <c r="J253" s="25" t="s">
         <v>377</v>
@@ -17458,11 +17506,11 @@
       </c>
       <c r="N253" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O253" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P253" s="8"/>
       <c r="Q253" s="50">
@@ -17555,8 +17603,8 @@
       <c r="H255" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I255" s="27">
-        <v>10.9</v>
+      <c r="I255" s="36">
+        <v>43.6</v>
       </c>
       <c r="J255" s="25" t="s">
         <v>377</v>
@@ -17570,11 +17618,11 @@
       </c>
       <c r="N255" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O255" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P255" s="8"/>
       <c r="Q255" s="50">
@@ -17611,8 +17659,8 @@
       <c r="H256" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I256" s="27">
-        <v>10.9</v>
+      <c r="I256" s="36">
+        <v>43.6</v>
       </c>
       <c r="J256" s="25" t="s">
         <v>377</v>
@@ -17626,11 +17674,11 @@
       </c>
       <c r="N256" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O256" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P256" s="8"/>
       <c r="Q256" s="50">
@@ -17667,8 +17715,8 @@
       <c r="H257" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I257" s="27">
-        <v>10.9</v>
+      <c r="I257" s="36">
+        <v>43.6</v>
       </c>
       <c r="J257" s="25" t="s">
         <v>377</v>
@@ -17682,11 +17730,11 @@
       </c>
       <c r="N257" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O257" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P257" s="8"/>
       <c r="Q257" s="50">
@@ -17723,8 +17771,8 @@
       <c r="H258" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I258" s="27">
-        <v>10.9</v>
+      <c r="I258" s="36">
+        <v>43.6</v>
       </c>
       <c r="J258" s="25" t="s">
         <v>377</v>
@@ -17738,11 +17786,11 @@
       </c>
       <c r="N258" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O258" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P258" s="8"/>
       <c r="Q258" s="50">
@@ -17779,8 +17827,8 @@
       <c r="H259" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I259" s="27">
-        <v>10.9</v>
+      <c r="I259" s="36">
+        <v>43.6</v>
       </c>
       <c r="J259" s="25" t="s">
         <v>377</v>
@@ -17794,11 +17842,11 @@
       </c>
       <c r="N259" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O259" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P259" s="8"/>
       <c r="Q259" s="50">
@@ -17835,8 +17883,8 @@
       <c r="H260" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I260" s="27">
-        <v>10.9</v>
+      <c r="I260" s="36">
+        <v>43.6</v>
       </c>
       <c r="J260" s="25" t="s">
         <v>377</v>
@@ -17850,11 +17898,11 @@
       </c>
       <c r="N260" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O260" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P260" s="8"/>
       <c r="Q260" s="50">
@@ -17947,8 +17995,8 @@
       <c r="H262" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I262" s="27">
-        <v>10.9</v>
+      <c r="I262" s="36">
+        <v>43.6</v>
       </c>
       <c r="J262" s="25" t="s">
         <v>377</v>
@@ -17962,11 +18010,11 @@
       </c>
       <c r="N262" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O262" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P262" s="8"/>
       <c r="Q262" s="50">
@@ -18003,8 +18051,8 @@
       <c r="H263" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I263" s="27">
-        <v>10.9</v>
+      <c r="I263" s="36">
+        <v>43.6</v>
       </c>
       <c r="J263" s="25" t="s">
         <v>377</v>
@@ -18018,11 +18066,11 @@
       </c>
       <c r="N263" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O263" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P263" s="8"/>
       <c r="Q263" s="50">
@@ -18059,8 +18107,8 @@
       <c r="H264" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I264" s="27">
-        <v>10.9</v>
+      <c r="I264" s="36">
+        <v>43.6</v>
       </c>
       <c r="J264" s="25" t="s">
         <v>377</v>
@@ -18074,11 +18122,11 @@
       </c>
       <c r="N264" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O264" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P264" s="8"/>
       <c r="Q264" s="50">
@@ -18115,8 +18163,8 @@
       <c r="H265" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I265" s="27">
-        <v>10.9</v>
+      <c r="I265" s="36">
+        <v>43.6</v>
       </c>
       <c r="J265" s="25" t="s">
         <v>377</v>
@@ -18130,11 +18178,11 @@
       </c>
       <c r="N265" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O265" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P265" s="8"/>
       <c r="Q265" s="50">
@@ -18171,8 +18219,8 @@
       <c r="H266" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I266" s="27">
-        <v>10.9</v>
+      <c r="I266" s="36">
+        <v>43.6</v>
       </c>
       <c r="J266" s="25" t="s">
         <v>377</v>
@@ -18186,11 +18234,11 @@
       </c>
       <c r="N266" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O266" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P266" s="8"/>
       <c r="Q266" s="50">
@@ -18227,8 +18275,8 @@
       <c r="H267" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I267" s="27">
-        <v>10.9</v>
+      <c r="I267" s="36">
+        <v>43.6</v>
       </c>
       <c r="J267" s="25" t="s">
         <v>377</v>
@@ -18242,11 +18290,11 @@
       </c>
       <c r="N267" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O267" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P267" s="8"/>
       <c r="Q267" s="50">
@@ -18339,8 +18387,8 @@
       <c r="H269" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I269" s="27">
-        <v>10.9</v>
+      <c r="I269" s="36">
+        <v>43.6</v>
       </c>
       <c r="J269" s="25" t="s">
         <v>377</v>
@@ -18354,11 +18402,11 @@
       </c>
       <c r="N269" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O269" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P269" s="8"/>
       <c r="Q269" s="50">
@@ -18395,8 +18443,8 @@
       <c r="H270" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I270" s="27">
-        <v>10.9</v>
+      <c r="I270" s="36">
+        <v>43.6</v>
       </c>
       <c r="J270" s="25" t="s">
         <v>377</v>
@@ -18410,11 +18458,11 @@
       </c>
       <c r="N270" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O270" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P270" s="8"/>
       <c r="Q270" s="50">
@@ -18451,8 +18499,8 @@
       <c r="H271" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I271" s="27">
-        <v>10.9</v>
+      <c r="I271" s="36">
+        <v>43.6</v>
       </c>
       <c r="J271" s="25" t="s">
         <v>377</v>
@@ -18466,11 +18514,11 @@
       </c>
       <c r="N271" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O271" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P271" s="8"/>
       <c r="Q271" s="50">
@@ -18507,8 +18555,8 @@
       <c r="H272" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I272" s="27">
-        <v>10.9</v>
+      <c r="I272" s="36">
+        <v>43.6</v>
       </c>
       <c r="J272" s="25" t="s">
         <v>377</v>
@@ -18522,11 +18570,11 @@
       </c>
       <c r="N272" s="30">
         <f t="shared" si="12"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O272" s="30">
         <f t="shared" si="13"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P272" s="8"/>
       <c r="Q272" s="50">
@@ -18563,8 +18611,8 @@
       <c r="H273" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I273" s="27">
-        <v>10.9</v>
+      <c r="I273" s="36">
+        <v>43.6</v>
       </c>
       <c r="J273" s="25" t="s">
         <v>377</v>
@@ -18578,11 +18626,11 @@
       </c>
       <c r="N273" s="30">
         <f t="shared" ref="N273:N281" si="16">I273*(1-M273)</f>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O273" s="30">
         <f t="shared" ref="O273:O290" si="17">N273*(1+J273)</f>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P273" s="8"/>
       <c r="Q273" s="50">
@@ -18619,8 +18667,8 @@
       <c r="H274" s="25" t="s">
         <v>191</v>
       </c>
-      <c r="I274" s="27">
-        <v>10.9</v>
+      <c r="I274" s="36">
+        <v>43.6</v>
       </c>
       <c r="J274" s="25" t="s">
         <v>377</v>
@@ -18634,11 +18682,11 @@
       </c>
       <c r="N274" s="30">
         <f t="shared" si="16"/>
-        <v>5.45</v>
+        <v>21.8</v>
       </c>
       <c r="O274" s="30">
         <f t="shared" si="17"/>
-        <v>5.6680000000000001</v>
+        <v>22.672000000000001</v>
       </c>
       <c r="P274" s="8"/>
       <c r="Q274" s="50">
@@ -18823,33 +18871,33 @@
         <v>177</v>
       </c>
       <c r="B278" s="16" t="s">
+        <v>700</v>
+      </c>
+      <c r="C278" s="16" t="s">
         <v>699</v>
       </c>
-      <c r="C278" s="16" t="s">
+      <c r="D278" s="31" t="s">
+        <v>697</v>
+      </c>
+      <c r="E278" s="94" t="s">
         <v>698</v>
       </c>
-      <c r="D278" s="31" t="s">
-        <v>696</v>
-      </c>
-      <c r="E278" s="31" t="s">
-        <v>697</v>
-      </c>
-      <c r="F278" s="32" t="s">
-        <v>699</v>
-      </c>
-      <c r="G278" s="32" t="s">
+      <c r="F278" s="95" t="s">
+        <v>700</v>
+      </c>
+      <c r="G278" s="95" t="s">
         <v>193</v>
       </c>
-      <c r="H278" s="32" t="s">
-        <v>191</v>
-      </c>
-      <c r="I278" s="33">
+      <c r="H278" s="95" t="s">
+        <v>191</v>
+      </c>
+      <c r="I278" s="96">
         <v>103.2</v>
       </c>
-      <c r="J278" s="32" t="s">
+      <c r="J278" s="95" t="s">
         <v>378</v>
       </c>
-      <c r="K278" s="34">
+      <c r="K278" s="38">
         <v>8052747326532</v>
       </c>
       <c r="L278" s="38" t="s">
@@ -18858,11 +18906,11 @@
       <c r="M278" s="29">
         <v>0.6</v>
       </c>
-      <c r="N278" s="23">
+      <c r="N278" s="92">
         <f t="shared" si="16"/>
         <v>41.28</v>
       </c>
-      <c r="O278" s="23">
+      <c r="O278" s="92">
         <f t="shared" si="17"/>
         <v>50.361600000000003</v>
       </c>
@@ -19222,35 +19270,35 @@
       <c r="D285" s="35">
         <v>1812</v>
       </c>
-      <c r="E285" s="35" t="s">
-        <v>695</v>
-      </c>
-      <c r="F285" s="35" t="s">
+      <c r="E285" s="87" t="s">
+        <v>696</v>
+      </c>
+      <c r="F285" s="87" t="s">
         <v>365</v>
       </c>
-      <c r="G285" s="25" t="s">
-        <v>191</v>
-      </c>
-      <c r="H285" s="25" t="s">
-        <v>191</v>
-      </c>
-      <c r="I285" s="36">
+      <c r="G285" s="89" t="s">
+        <v>191</v>
+      </c>
+      <c r="H285" s="89" t="s">
+        <v>191</v>
+      </c>
+      <c r="I285" s="90">
         <v>75</v>
       </c>
-      <c r="J285" s="25" t="s">
+      <c r="J285" s="89" t="s">
         <v>378</v>
       </c>
-      <c r="K285" s="37">
+      <c r="K285" s="91">
         <v>8058032048615</v>
       </c>
-      <c r="L285" s="37"/>
-      <c r="M285" s="37" t="s">
+      <c r="L285" s="91"/>
+      <c r="M285" s="91" t="s">
         <v>683</v>
       </c>
-      <c r="N285" s="36">
+      <c r="N285" s="90">
         <v>75</v>
       </c>
-      <c r="O285" s="30">
+      <c r="O285" s="92">
         <f t="shared" si="17"/>
         <v>91.5</v>
       </c>
@@ -19333,7 +19381,7 @@
         <v>1781</v>
       </c>
       <c r="E287" s="16" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="F287" s="16" t="s">
         <v>365</v>
@@ -19351,7 +19399,7 @@
         <v>378</v>
       </c>
       <c r="K287" s="16" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="L287" s="16"/>
       <c r="M287" s="16" t="s">
@@ -19388,7 +19436,7 @@
         <v>1783</v>
       </c>
       <c r="E288" s="16" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="F288" s="16" t="s">
         <v>365</v>
@@ -19406,7 +19454,7 @@
         <v>378</v>
       </c>
       <c r="K288" s="16" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="L288" s="16"/>
       <c r="M288" s="16" t="s">
@@ -19442,35 +19490,35 @@
       <c r="D289" s="16">
         <v>1813</v>
       </c>
-      <c r="E289" s="16" t="s">
-        <v>706</v>
-      </c>
-      <c r="F289" s="16" t="s">
+      <c r="E289" s="88" t="s">
+        <v>707</v>
+      </c>
+      <c r="F289" s="88" t="s">
         <v>365</v>
       </c>
-      <c r="G289" s="16">
+      <c r="G289" s="88">
         <v>1</v>
       </c>
-      <c r="H289" s="16">
+      <c r="H289" s="88">
         <v>1</v>
       </c>
-      <c r="I289" s="36">
+      <c r="I289" s="90">
         <v>75</v>
       </c>
-      <c r="J289" s="16" t="s">
+      <c r="J289" s="88" t="s">
         <v>378</v>
       </c>
-      <c r="K289" s="52">
+      <c r="K289" s="93">
         <v>8058032048622</v>
       </c>
-      <c r="L289" s="16"/>
-      <c r="M289" s="16" t="s">
+      <c r="L289" s="88"/>
+      <c r="M289" s="88" t="s">
         <v>683</v>
       </c>
-      <c r="N289" s="36">
+      <c r="N289" s="90">
         <v>75</v>
       </c>
-      <c r="O289" s="30">
+      <c r="O289" s="92">
         <f t="shared" si="17"/>
         <v>91.5</v>
       </c>
@@ -19498,7 +19546,7 @@
         <v>1590</v>
       </c>
       <c r="E290" s="16" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="F290" s="16" t="s">
         <v>365</v>
@@ -19516,7 +19564,7 @@
         <v>378</v>
       </c>
       <c r="K290" s="16" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="L290" s="16"/>
       <c r="M290" s="16" t="s">
@@ -19597,14 +19645,14 @@
       <c r="K293" s="43"/>
       <c r="L293" s="43"/>
       <c r="M293" s="43"/>
-      <c r="N293" s="83" t="s">
-        <v>689</v>
-      </c>
-      <c r="O293" s="84"/>
-      <c r="Q293" s="65" t="s">
-        <v>693</v>
-      </c>
-      <c r="R293" s="68">
+      <c r="N293" s="55" t="s">
+        <v>690</v>
+      </c>
+      <c r="O293" s="56"/>
+      <c r="Q293" s="60" t="s">
+        <v>694</v>
+      </c>
+      <c r="R293" s="63">
         <f>R291+N297</f>
         <v>11.59</v>
       </c>
@@ -19630,8 +19678,8 @@
         <f>MIN(MAX(Q291*N294,9.5),99)</f>
         <v>9.5</v>
       </c>
-      <c r="Q294" s="66"/>
-      <c r="R294" s="69"/>
+      <c r="Q294" s="61"/>
+      <c r="R294" s="64"/>
     </row>
     <row r="295" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A295" s="43"/>
@@ -19647,12 +19695,12 @@
       <c r="K295" s="43"/>
       <c r="L295" s="43"/>
       <c r="M295" s="43"/>
-      <c r="N295" s="85" t="s">
-        <v>692</v>
-      </c>
-      <c r="O295" s="86"/>
-      <c r="Q295" s="66"/>
-      <c r="R295" s="69"/>
+      <c r="N295" s="57" t="s">
+        <v>693</v>
+      </c>
+      <c r="O295" s="58"/>
+      <c r="Q295" s="61"/>
+      <c r="R295" s="64"/>
     </row>
     <row r="296" spans="1:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A296" s="43"/>
@@ -19675,8 +19723,8 @@
         <f>O294*N296</f>
         <v>2.09</v>
       </c>
-      <c r="Q296" s="67"/>
-      <c r="R296" s="70"/>
+      <c r="Q296" s="62"/>
+      <c r="R296" s="65"/>
     </row>
     <row r="297" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A297" s="43"/>
@@ -19692,29 +19740,14 @@
       <c r="K297" s="43"/>
       <c r="L297" s="43"/>
       <c r="M297" s="43"/>
-      <c r="N297" s="87">
+      <c r="N297" s="59">
         <f>O294+O296</f>
         <v>11.59</v>
       </c>
-      <c r="O297" s="87"/>
+      <c r="O297" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="I7:P7"/>
-    <mergeCell ref="I6:P6"/>
-    <mergeCell ref="N293:O293"/>
-    <mergeCell ref="N295:O295"/>
-    <mergeCell ref="N297:O297"/>
-    <mergeCell ref="Q293:Q296"/>
-    <mergeCell ref="R293:R296"/>
-    <mergeCell ref="D12:G12"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="D8:G8"/>
-    <mergeCell ref="H8:H12"/>
-    <mergeCell ref="I8:P12"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="D10:G10"/>
     <mergeCell ref="A2:P2"/>
     <mergeCell ref="A13:P13"/>
     <mergeCell ref="A7:C7"/>
@@ -19731,6 +19764,21 @@
     <mergeCell ref="D11:G11"/>
     <mergeCell ref="D7:G7"/>
     <mergeCell ref="A12:C12"/>
+    <mergeCell ref="Q293:Q296"/>
+    <mergeCell ref="R293:R296"/>
+    <mergeCell ref="D12:G12"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="H8:H12"/>
+    <mergeCell ref="I8:P12"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="D10:G10"/>
+    <mergeCell ref="I7:P7"/>
+    <mergeCell ref="I6:P6"/>
+    <mergeCell ref="N293:O293"/>
+    <mergeCell ref="N295:O295"/>
+    <mergeCell ref="N297:O297"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>